<commit_message>
Atualização de layout/texto — 16/05/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -401,6 +401,706 @@
         <is>
           <t>pct_uti</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Uniflor</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>189.9</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Santo Inacio</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>9</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>139.3</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>22.2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nova Esperanca</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>36</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>132.6</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Itaguaje</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>110.4</v>
+      </c>
+      <c r="F5">
+        <v>22.1</v>
+      </c>
+      <c r="G5">
+        <v>20</v>
+      </c>
+      <c r="H5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Nossa Senhora Das Gracas</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>109</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sao Jorge Do Ivai</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7">
+        <v>96.7</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Maringa</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>346</v>
+      </c>
+      <c r="C8">
+        <v>25</v>
+      </c>
+      <c r="D8">
+        <v>98</v>
+      </c>
+      <c r="E8">
+        <v>80.5</v>
+      </c>
+      <c r="F8">
+        <v>5.8</v>
+      </c>
+      <c r="G8">
+        <v>7.2</v>
+      </c>
+      <c r="H8">
+        <v>28.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Colorado</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>17</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Itambe</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>4</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>64.2</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ourizona</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>62.6</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Florai</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>62.4</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Santa Ines</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>57.3</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Marialva</t>
+        </is>
+      </c>
+      <c r="B14">
+        <v>25</v>
+      </c>
+      <c r="C14">
+        <v>2</v>
+      </c>
+      <c r="D14">
+        <v>13</v>
+      </c>
+      <c r="E14">
+        <v>55.9</v>
+      </c>
+      <c r="F14">
+        <v>4.5</v>
+      </c>
+      <c r="G14">
+        <v>8</v>
+      </c>
+      <c r="H14">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Paranacity</t>
+        </is>
+      </c>
+      <c r="B15">
+        <v>5</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>52.4</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sarandi</t>
+        </is>
+      </c>
+      <c r="B16">
+        <v>58</v>
+      </c>
+      <c r="C16">
+        <v>4</v>
+      </c>
+      <c r="D16">
+        <v>25</v>
+      </c>
+      <c r="E16">
+        <v>45.3</v>
+      </c>
+      <c r="F16">
+        <v>3.1</v>
+      </c>
+      <c r="G16">
+        <v>6.9</v>
+      </c>
+      <c r="H16">
+        <v>43.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mandaguacu</t>
+        </is>
+      </c>
+      <c r="B17">
+        <v>14</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <v>5</v>
+      </c>
+      <c r="E17">
+        <v>40.6</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>35.7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="B18">
+        <v>4</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>3</v>
+      </c>
+      <c r="E18">
+        <v>34.1</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Paicandu</t>
+        </is>
+      </c>
+      <c r="B19">
+        <v>15</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
+        <v>7</v>
+      </c>
+      <c r="E19">
+        <v>30.8</v>
+      </c>
+      <c r="F19">
+        <v>2.1</v>
+      </c>
+      <c r="G19">
+        <v>6.7</v>
+      </c>
+      <c r="H19">
+        <v>46.7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Atalaia</t>
+        </is>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>24.7</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Munhoz De Melo</t>
+        </is>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>24.6</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Lobato</t>
+        </is>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>21.2</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Iguaracu</t>
+        </is>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>17.6</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Mandaguari</t>
+        </is>
+      </c>
+      <c r="B24">
+        <v>6</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>4</v>
+      </c>
+      <c r="E24">
+        <v>15.7</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Astorga</t>
+        </is>
+      </c>
+      <c r="B25">
+        <v>4</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>15.3</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Doutor Camargo</t>
+        </is>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>15.3</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -410,7 +1110,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -428,6 +1128,201 @@
         <is>
           <t>n_total</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Obesidade</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>57.7</v>
+      </c>
+      <c r="C2">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cardiopatia</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>57.9</v>
+      </c>
+      <c r="C3">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Diabetes</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>57.9</v>
+      </c>
+      <c r="C4">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Imunodepressão</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>57.9</v>
+      </c>
+      <c r="C5">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Evolução (Desfecho)</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>60.3</v>
+      </c>
+      <c r="C6">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Critério Confirmação</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>82.7</v>
+      </c>
+      <c r="C7">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bairro</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>91.09999999999999</v>
+      </c>
+      <c r="C8">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Antiviral</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>96.5</v>
+      </c>
+      <c r="C9">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Data Internação</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>97.2</v>
+      </c>
+      <c r="C10">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Raça/Cor</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>99.8</v>
+      </c>
+      <c r="C11">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Vacinação COVID</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>99.8</v>
+      </c>
+      <c r="C12">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sexo</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>100</v>
+      </c>
+      <c r="C13">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Idade</t>
+        </is>
+      </c>
+      <c r="B14">
+        <v>100</v>
+      </c>
+      <c r="C14">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Semana Epidemiológica</t>
+        </is>
+      </c>
+      <c r="B15">
+        <v>100</v>
+      </c>
+      <c r="C15">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Data Início Sintomas</t>
+        </is>
+      </c>
+      <c r="B16">
+        <v>100</v>
+      </c>
+      <c r="C16">
+        <v>572</v>
       </c>
     </row>
   </sheetData>
@@ -437,7 +1332,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -455,6 +1350,136 @@
         <is>
           <t>pct</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cardiopatia</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>147</v>
+      </c>
+      <c r="C2">
+        <v>25.7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Diabetes</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>75</v>
+      </c>
+      <c r="C3">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Doença Neurológica</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>69</v>
+      </c>
+      <c r="C4">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Asma</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>67</v>
+      </c>
+      <c r="C5">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pneumopatia</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>48</v>
+      </c>
+      <c r="C6">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Obesidade</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>13</v>
+      </c>
+      <c r="C7">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Imunodepressão</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>13</v>
+      </c>
+      <c r="C8">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Doença Renal</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>12</v>
+      </c>
+      <c r="C9">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Doença Hepática</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>7</v>
+      </c>
+      <c r="C10">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Síndrome de Down</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>6</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -464,7 +1489,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -487,6 +1512,166 @@
         <is>
           <t>letalidade_pct</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0-6 meses</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>47</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1-4 anos</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>107</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>10-14 anos</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>20-29 anos</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>12</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>30-39 anos</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>6.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>40-49 anos</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>5-9 anos</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>46</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>50-59 anos</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>32</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6-11 meses</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>48</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>60 anos e mais</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>221</v>
+      </c>
+      <c r="C11">
+        <v>27</v>
+      </c>
+      <c r="D11">
+        <v>12.2</v>
       </c>
     </row>
   </sheetData>
@@ -496,7 +1681,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -519,6 +1704,166 @@
         <is>
           <t>pct_uti</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0-6 meses</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>47</v>
+      </c>
+      <c r="C2">
+        <v>22</v>
+      </c>
+      <c r="D2">
+        <v>46.8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1-4 anos</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>107</v>
+      </c>
+      <c r="C3">
+        <v>15</v>
+      </c>
+      <c r="D3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>10-14 anos</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>31.2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>20-29 anos</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>12</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>30-39 anos</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>26.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>40-49 anos</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>10</v>
+      </c>
+      <c r="D7">
+        <v>41.7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>5-9 anos</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>46</v>
+      </c>
+      <c r="C8">
+        <v>14</v>
+      </c>
+      <c r="D8">
+        <v>30.4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>50-59 anos</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>32</v>
+      </c>
+      <c r="C9">
+        <v>14</v>
+      </c>
+      <c r="D9">
+        <v>43.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6-11 meses</t>
+        </is>
+      </c>
+      <c r="B10">
+        <v>48</v>
+      </c>
+      <c r="C10">
+        <v>8</v>
+      </c>
+      <c r="D10">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>60 anos e mais</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>221</v>
+      </c>
+      <c r="C11">
+        <v>73</v>
+      </c>
+      <c r="D11">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +1873,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -546,6 +1891,45 @@
         <is>
           <t>pct</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Laboratorial</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>252</v>
+      </c>
+      <c r="C2">
+        <v>98.40000000000001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Clínico-Imagem</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Não informado</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>
@@ -555,7 +1939,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -573,6 +1957,45 @@
         <is>
           <t>pct</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ignorado/Não registrado</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>20</v>
+      </c>
+      <c r="C2">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>460</v>
+      </c>
+      <c r="C3">
+        <v>80.40000000000001</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>92</v>
+      </c>
+      <c r="C4">
+        <v>16.1</v>
       </c>
     </row>
   </sheetData>
@@ -582,7 +2005,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -602,6 +2025,45 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ignorado/Não registrado</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Não vacinado</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>248</v>
+      </c>
+      <c r="C3">
+        <v>43.4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Vacinado</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>323</v>
+      </c>
+      <c r="C4">
+        <v>56.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização de dados — 10/06/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -410,7 +410,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -419,7 +419,7 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>189.9</v>
+        <v>237.4</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -434,20 +434,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Santo Inacio</t>
+          <t>Nova Esperanca</t>
         </is>
       </c>
       <c r="B3">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>139.3</v>
+        <v>206.3</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -456,26 +456,26 @@
         <v>0</v>
       </c>
       <c r="H3">
-        <v>22.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nova Esperanca</t>
+          <t>Nossa Senhora Das Gracas</t>
         </is>
       </c>
       <c r="B4">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
-        <v>132.6</v>
+        <v>163.5</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -484,32 +484,32 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>5.6</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Itaguaje</t>
+          <t>Santo Inacio</t>
         </is>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5">
-        <v>110.4</v>
+        <v>154.7</v>
       </c>
       <c r="F5">
-        <v>22.1</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H5">
         <v>20</v>
@@ -518,48 +518,48 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nossa Senhora Das Gracas</t>
+          <t>Itaguaje</t>
         </is>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6">
-        <v>109</v>
+        <v>154.5</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>22.1</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="H6">
-        <v>50</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sao Jorge Do Ivai</t>
+          <t>Ourizona</t>
         </is>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C7">
         <v>0</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7">
-        <v>96.7</v>
+        <v>125.3</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -568,82 +568,82 @@
         <v>0</v>
       </c>
       <c r="H7">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Maringa</t>
+          <t>Atalaia</t>
         </is>
       </c>
       <c r="B8">
-        <v>346</v>
+        <v>5</v>
       </c>
       <c r="C8">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>80.5</v>
+        <v>123.6</v>
       </c>
       <c r="F8">
-        <v>5.8</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>7.2</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>28.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Colorado</t>
+          <t>Maringa</t>
         </is>
       </c>
       <c r="B9">
-        <v>17</v>
+        <v>506</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>142</v>
       </c>
       <c r="E9">
-        <v>72.90000000000001</v>
+        <v>117.8</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>8.1</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="H9">
-        <v>5.9</v>
+        <v>28.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Itambe</t>
+          <t>Sao Jorge Do Ivai</t>
         </is>
       </c>
       <c r="B10">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C10">
         <v>0</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10">
-        <v>64.2</v>
+        <v>116.1</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -652,26 +652,26 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>25</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ourizona</t>
+          <t>Colorado</t>
         </is>
       </c>
       <c r="B11">
+        <v>24</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
         <v>2</v>
       </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
       <c r="E11">
-        <v>62.6</v>
+        <v>102.9</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -680,54 +680,54 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Florai</t>
+          <t>Marialva</t>
         </is>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E12">
-        <v>62.4</v>
+        <v>69.3</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="H12">
-        <v>33.3</v>
+        <v>51.6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Santa Ines</t>
+          <t>Itambe</t>
         </is>
       </c>
       <c r="B13">
+        <v>4</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
         <v>1</v>
       </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
       <c r="E13">
-        <v>57.3</v>
+        <v>64.2</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -736,45 +736,45 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Marialva</t>
+          <t>Paranacity</t>
         </is>
       </c>
       <c r="B14">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="C14">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D14">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E14">
-        <v>55.9</v>
+        <v>62.8</v>
       </c>
       <c r="F14">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H14">
-        <v>52</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Paranacity</t>
+          <t>Florai</t>
         </is>
       </c>
       <c r="B15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -783,7 +783,7 @@
         <v>1</v>
       </c>
       <c r="E15">
-        <v>52.4</v>
+        <v>62.4</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -792,82 +792,82 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>20</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sarandi</t>
+          <t>Santa Ines</t>
         </is>
       </c>
       <c r="B16">
-        <v>58</v>
+        <v>1</v>
       </c>
       <c r="C16">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>45.3</v>
+        <v>57.3</v>
       </c>
       <c r="F16">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>6.9</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>43.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mandaguacu</t>
+          <t>Sarandi</t>
         </is>
       </c>
       <c r="B17">
-        <v>14</v>
+        <v>73</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D17">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="E17">
-        <v>40.6</v>
+        <v>57</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>3.9</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="H17">
-        <v>35.7</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Lobato</t>
         </is>
       </c>
       <c r="B18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C18">
         <v>0</v>
       </c>
       <c r="D18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E18">
-        <v>34.1</v>
+        <v>42.5</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -876,82 +876,82 @@
         <v>0</v>
       </c>
       <c r="H18">
-        <v>75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Paicandu</t>
+          <t>Mandaguacu</t>
         </is>
       </c>
       <c r="B19">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E19">
-        <v>30.8</v>
+        <v>40.6</v>
       </c>
       <c r="F19">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>6.7</v>
+        <v>0</v>
       </c>
       <c r="H19">
-        <v>46.7</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Atalaia</t>
+          <t>Paicandu</t>
         </is>
       </c>
       <c r="B20">
+        <v>18</v>
+      </c>
+      <c r="C20">
         <v>1</v>
       </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
       <c r="D20">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E20">
-        <v>24.7</v>
+        <v>37</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>5.6</v>
       </c>
       <c r="H20">
-        <v>0</v>
+        <v>55.6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Munhoz De Melo</t>
+          <t>Floresta</t>
         </is>
       </c>
       <c r="B21">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>24.6</v>
+        <v>34.7</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -960,26 +960,26 @@
         <v>0</v>
       </c>
       <c r="H21">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Lobato</t>
+          <t>Astorga</t>
         </is>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C22">
         <v>0</v>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E22">
-        <v>21.2</v>
+        <v>34.3</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -988,26 +988,26 @@
         <v>0</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Iguaracu</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="B23">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C23">
         <v>0</v>
       </c>
       <c r="D23">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E23">
-        <v>17.6</v>
+        <v>34.1</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -1016,26 +1016,26 @@
         <v>0</v>
       </c>
       <c r="H23">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mandaguari</t>
+          <t>Munhoz De Melo</t>
         </is>
       </c>
       <c r="B24">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C24">
         <v>0</v>
       </c>
       <c r="D24">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E24">
-        <v>15.7</v>
+        <v>24.6</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -1044,26 +1044,26 @@
         <v>0</v>
       </c>
       <c r="H24">
-        <v>66.7</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Astorga</t>
+          <t>Mandaguari</t>
         </is>
       </c>
       <c r="B25">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E25">
-        <v>15.3</v>
+        <v>18.3</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1072,13 +1072,13 @@
         <v>0</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>71.40000000000001</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Doutor Camargo</t>
+          <t>Iguaracu</t>
         </is>
       </c>
       <c r="B26">
@@ -1088,18 +1088,46 @@
         <v>0</v>
       </c>
       <c r="D26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26">
+        <v>17.6</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Doutor Camargo</t>
+        </is>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
         <v>15.3</v>
       </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
-      <c r="G26">
-        <v>0</v>
-      </c>
-      <c r="H26">
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
         <v>0</v>
       </c>
     </row>
@@ -1137,36 +1165,36 @@
         </is>
       </c>
       <c r="B2">
-        <v>57.7</v>
+        <v>54.8</v>
       </c>
       <c r="C2">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cardiopatia</t>
+          <t>Diabetes</t>
         </is>
       </c>
       <c r="B3">
-        <v>57.9</v>
+        <v>55</v>
       </c>
       <c r="C3">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Diabetes</t>
+          <t>Cardiopatia</t>
         </is>
       </c>
       <c r="B4">
-        <v>57.9</v>
+        <v>55.1</v>
       </c>
       <c r="C4">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="5">
@@ -1176,10 +1204,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>57.9</v>
+        <v>55.1</v>
       </c>
       <c r="C5">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="6">
@@ -1189,10 +1217,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>60.3</v>
+        <v>59.2</v>
       </c>
       <c r="C6">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="7">
@@ -1202,10 +1230,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>82.7</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="C7">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="8">
@@ -1215,36 +1243,36 @@
         </is>
       </c>
       <c r="B8">
-        <v>91.09999999999999</v>
+        <v>90.5</v>
       </c>
       <c r="C8">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Antiviral</t>
+          <t>Data Internação</t>
         </is>
       </c>
       <c r="B9">
-        <v>96.5</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="C9">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Data Internação</t>
+          <t>Antiviral</t>
         </is>
       </c>
       <c r="B10">
-        <v>97.2</v>
+        <v>95.5</v>
       </c>
       <c r="C10">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="11">
@@ -1254,10 +1282,10 @@
         </is>
       </c>
       <c r="B11">
-        <v>99.8</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="C11">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="12">
@@ -1270,7 +1298,7 @@
         <v>99.8</v>
       </c>
       <c r="C12">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="13">
@@ -1283,7 +1311,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="14">
@@ -1296,7 +1324,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="15">
@@ -1309,7 +1337,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
     <row r="16">
@@ -1322,7 +1350,7 @@
         <v>100</v>
       </c>
       <c r="C16">
-        <v>572</v>
+        <v>808</v>
       </c>
     </row>
   </sheetData>
@@ -1332,7 +1360,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1359,10 +1387,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>147</v>
+        <v>191</v>
       </c>
       <c r="C2">
-        <v>25.7</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="3">
@@ -1372,36 +1400,36 @@
         </is>
       </c>
       <c r="B3">
-        <v>75</v>
+        <v>104</v>
       </c>
       <c r="C3">
-        <v>13.1</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Doença Neurológica</t>
+          <t>Asma</t>
         </is>
       </c>
       <c r="B4">
-        <v>69</v>
+        <v>103</v>
       </c>
       <c r="C4">
-        <v>12.1</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Asma</t>
+          <t>Doença Neurológica</t>
         </is>
       </c>
       <c r="B5">
-        <v>67</v>
+        <v>92</v>
       </c>
       <c r="C5">
-        <v>11.7</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="6">
@@ -1411,23 +1439,23 @@
         </is>
       </c>
       <c r="B6">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="C6">
-        <v>8.4</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Obesidade</t>
+          <t>Doença Renal</t>
         </is>
       </c>
       <c r="B7">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C7">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="8">
@@ -1437,23 +1465,23 @@
         </is>
       </c>
       <c r="B8">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C8">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Doença Renal</t>
+          <t>Obesidade</t>
         </is>
       </c>
       <c r="B9">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C9">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1463,10 +1491,10 @@
         </is>
       </c>
       <c r="B10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C10">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1476,10 +1504,23 @@
         </is>
       </c>
       <c r="B11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C11">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Puérpera</t>
+        </is>
+      </c>
+      <c r="B12">
         <v>1</v>
+      </c>
+      <c r="C12">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -1489,7 +1530,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1521,7 +1562,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1537,7 +1578,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>107</v>
+        <v>151</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1553,7 +1594,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1565,113 +1606,129 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20-29 anos</t>
+          <t>15-19 anos</t>
         </is>
       </c>
       <c r="B5">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>30-39 anos</t>
+          <t>20-29 anos</t>
         </is>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>6.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>40-49 anos</t>
+          <t>30-39 anos</t>
         </is>
       </c>
       <c r="B7">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7">
-        <v>4.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5-9 anos</t>
+          <t>40-49 anos</t>
         </is>
       </c>
       <c r="B8">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8">
-        <v>2.2</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>50-59 anos</t>
+          <t>5-9 anos</t>
         </is>
       </c>
       <c r="B9">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9">
-        <v>6.2</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6-11 meses</t>
+          <t>50-59 anos</t>
         </is>
       </c>
       <c r="B10">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>6-11 meses</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>79</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>60 anos e mais</t>
         </is>
       </c>
-      <c r="B11">
-        <v>221</v>
-      </c>
-      <c r="C11">
-        <v>27</v>
-      </c>
-      <c r="D11">
-        <v>12.2</v>
+      <c r="B12">
+        <v>302</v>
+      </c>
+      <c r="C12">
+        <v>35</v>
+      </c>
+      <c r="D12">
+        <v>11.6</v>
       </c>
     </row>
   </sheetData>
@@ -1681,7 +1738,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1713,13 +1770,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="C2">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="D2">
-        <v>46.8</v>
+        <v>45.6</v>
       </c>
     </row>
     <row r="3">
@@ -1729,13 +1786,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>107</v>
+        <v>151</v>
       </c>
       <c r="C3">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D3">
-        <v>14</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="4">
@@ -1745,125 +1802,141 @@
         </is>
       </c>
       <c r="B4">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>31.2</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20-29 anos</t>
+          <t>15-19 anos</t>
         </is>
       </c>
       <c r="B5">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5">
-        <v>33.3</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>30-39 anos</t>
+          <t>20-29 anos</t>
         </is>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
       <c r="D6">
-        <v>26.7</v>
+        <v>30.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>40-49 anos</t>
+          <t>30-39 anos</t>
         </is>
       </c>
       <c r="B7">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C7">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D7">
-        <v>41.7</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5-9 anos</t>
+          <t>40-49 anos</t>
         </is>
       </c>
       <c r="B8">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="C8">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D8">
-        <v>30.4</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>50-59 anos</t>
+          <t>5-9 anos</t>
         </is>
       </c>
       <c r="B9">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="C9">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D9">
-        <v>43.8</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6-11 meses</t>
+          <t>50-59 anos</t>
         </is>
       </c>
       <c r="B10">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C10">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D10">
-        <v>16.7</v>
+        <v>43.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>6-11 meses</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>79</v>
+      </c>
+      <c r="C11">
+        <v>18</v>
+      </c>
+      <c r="D11">
+        <v>22.8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>60 anos e mais</t>
         </is>
       </c>
-      <c r="B11">
-        <v>221</v>
-      </c>
-      <c r="C11">
-        <v>73</v>
-      </c>
-      <c r="D11">
-        <v>33</v>
+      <c r="B12">
+        <v>302</v>
+      </c>
+      <c r="C12">
+        <v>93</v>
+      </c>
+      <c r="D12">
+        <v>30.8</v>
       </c>
     </row>
   </sheetData>
@@ -1900,36 +1973,36 @@
         </is>
       </c>
       <c r="B2">
-        <v>252</v>
+        <v>355</v>
       </c>
       <c r="C2">
-        <v>98.40000000000001</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Clínico-Imagem</t>
+          <t>Não informado</t>
         </is>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C3">
-        <v>0.8</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Não informado</t>
+          <t>Clínico-Imagem</t>
         </is>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
       <c r="C4">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>
@@ -1966,10 +2039,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="C2">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="3">
@@ -1979,10 +2052,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>460</v>
+        <v>608</v>
       </c>
       <c r="C3">
-        <v>80.40000000000001</v>
+        <v>75.2</v>
       </c>
     </row>
     <row r="4">
@@ -1992,10 +2065,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>92</v>
+        <v>164</v>
       </c>
       <c r="C4">
-        <v>16.1</v>
+        <v>20.3</v>
       </c>
     </row>
   </sheetData>
@@ -2032,7 +2105,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2">
         <v>0.2</v>
@@ -2045,10 +2118,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>248</v>
+        <v>367</v>
       </c>
       <c r="C3">
-        <v>43.4</v>
+        <v>45.4</v>
       </c>
     </row>
     <row r="4">
@@ -2058,10 +2131,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>323</v>
+        <v>439</v>
       </c>
       <c r="C4">
-        <v>56.5</v>
+        <v>54.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização de dados — 17/06/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -438,16 +438,16 @@
         </is>
       </c>
       <c r="B3">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3">
-        <v>206.3</v>
+        <v>232.1</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -456,26 +456,26 @@
         <v>0</v>
       </c>
       <c r="H3">
-        <v>5.4</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nossa Senhora Das Gracas</t>
+          <t>Atalaia</t>
         </is>
       </c>
       <c r="B4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>163.5</v>
+        <v>173</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -484,26 +484,26 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Santo Inacio</t>
+          <t>Nossa Senhora Das Gracas</t>
         </is>
       </c>
       <c r="B5">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5">
-        <v>154.7</v>
+        <v>163.5</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -512,82 +512,82 @@
         <v>0</v>
       </c>
       <c r="H5">
-        <v>20</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Itaguaje</t>
+          <t>Santo Inacio</t>
         </is>
       </c>
       <c r="B6">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>154.5</v>
+        <v>154.7</v>
       </c>
       <c r="F6">
-        <v>22.1</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>14.3</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>14.3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ourizona</t>
+          <t>Itaguaje</t>
         </is>
       </c>
       <c r="B7">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7">
-        <v>125.3</v>
+        <v>154.5</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>22.1</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="H7">
-        <v>25</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atalaia</t>
+          <t>Sao Jorge Do Ivai</t>
         </is>
       </c>
       <c r="B8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E8">
-        <v>123.6</v>
+        <v>135.4</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -596,7 +596,7 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="9">
@@ -606,44 +606,44 @@
         </is>
       </c>
       <c r="B9">
-        <v>506</v>
+        <v>556</v>
       </c>
       <c r="C9">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D9">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="E9">
-        <v>117.8</v>
+        <v>129.4</v>
       </c>
       <c r="F9">
-        <v>8.1</v>
+        <v>9.1</v>
       </c>
       <c r="G9">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="H9">
-        <v>28.1</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sao Jorge Do Ivai</t>
+          <t>Ourizona</t>
         </is>
       </c>
       <c r="B10">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C10">
         <v>0</v>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E10">
-        <v>116.1</v>
+        <v>125.3</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -652,7 +652,7 @@
         <v>0</v>
       </c>
       <c r="H10">
-        <v>50</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>2</v>
       </c>
       <c r="E11">
-        <v>102.9</v>
+        <v>111.5</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -680,63 +680,63 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>8.300000000000001</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Marialva</t>
+          <t>Florai</t>
         </is>
       </c>
       <c r="B12">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D12">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E12">
-        <v>69.3</v>
+        <v>83.2</v>
       </c>
       <c r="F12">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>6.5</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>51.6</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Itambe</t>
+          <t>Marialva</t>
         </is>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E13">
-        <v>64.2</v>
+        <v>76</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="H13">
-        <v>25</v>
+        <v>47.1</v>
       </c>
     </row>
     <row r="14">
@@ -746,7 +746,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -755,7 +755,7 @@
         <v>1</v>
       </c>
       <c r="E14">
-        <v>62.8</v>
+        <v>73.3</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -764,17 +764,17 @@
         <v>0</v>
       </c>
       <c r="H14">
-        <v>16.7</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Florai</t>
+          <t>Itambe</t>
         </is>
       </c>
       <c r="B15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -783,7 +783,7 @@
         <v>1</v>
       </c>
       <c r="E15">
-        <v>62.4</v>
+        <v>64.2</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -792,63 +792,63 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>33.3</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Santa Ines</t>
+          <t>Sarandi</t>
         </is>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>79</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D16">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E16">
-        <v>57.3</v>
+        <v>61.7</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>3.9</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>6.3</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>41.8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sarandi</t>
+          <t>Santa Ines</t>
         </is>
       </c>
       <c r="B17">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="C17">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D17">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E17">
-        <v>57</v>
+        <v>57.3</v>
       </c>
       <c r="F17">
-        <v>3.9</v>
+        <v>0</v>
       </c>
       <c r="G17">
-        <v>6.8</v>
+        <v>0</v>
       </c>
       <c r="H17">
-        <v>42.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -910,76 +910,76 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Paicandu</t>
+          <t>Astorga</t>
         </is>
       </c>
       <c r="B20">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E20">
-        <v>37</v>
+        <v>38.2</v>
       </c>
       <c r="F20">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>5.6</v>
+        <v>0</v>
       </c>
       <c r="H20">
-        <v>55.6</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Floresta</t>
+          <t>Paicandu</t>
         </is>
       </c>
       <c r="B21">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E21">
-        <v>34.7</v>
+        <v>37</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>5.6</v>
       </c>
       <c r="H21">
-        <v>0</v>
+        <v>55.6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Astorga</t>
+          <t>Floresta</t>
         </is>
       </c>
       <c r="B22">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C22">
         <v>0</v>
       </c>
       <c r="D22">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E22">
-        <v>34.3</v>
+        <v>34.7</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -988,7 +988,7 @@
         <v>0</v>
       </c>
       <c r="H22">
-        <v>33.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1054,16 +1054,16 @@
         </is>
       </c>
       <c r="B25">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E25">
-        <v>18.3</v>
+        <v>20.9</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1072,7 +1072,7 @@
         <v>0</v>
       </c>
       <c r="H25">
-        <v>71.40000000000001</v>
+        <v>75</v>
       </c>
     </row>
     <row r="26">
@@ -1165,10 +1165,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>54.8</v>
+        <v>56.4</v>
       </c>
       <c r="C2">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="3">
@@ -1178,10 +1178,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>55</v>
+        <v>56.5</v>
       </c>
       <c r="C3">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="4">
@@ -1191,10 +1191,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>55.1</v>
+        <v>56.6</v>
       </c>
       <c r="C4">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="5">
@@ -1204,10 +1204,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>55.1</v>
+        <v>56.6</v>
       </c>
       <c r="C5">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="6">
@@ -1217,10 +1217,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>59.2</v>
+        <v>61.5</v>
       </c>
       <c r="C6">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="7">
@@ -1230,10 +1230,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>73.90000000000001</v>
+        <v>77.3</v>
       </c>
       <c r="C7">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="8">
@@ -1243,10 +1243,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>90.5</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="C8">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="9">
@@ -1256,10 +1256,10 @@
         </is>
       </c>
       <c r="B9">
-        <v>94.09999999999999</v>
+        <v>94.5</v>
       </c>
       <c r="C9">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="10">
@@ -1269,10 +1269,10 @@
         </is>
       </c>
       <c r="B10">
-        <v>95.5</v>
+        <v>97.5</v>
       </c>
       <c r="C10">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="11">
@@ -1282,10 +1282,10 @@
         </is>
       </c>
       <c r="B11">
-        <v>99.59999999999999</v>
+        <v>99.7</v>
       </c>
       <c r="C11">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="12">
@@ -1298,7 +1298,7 @@
         <v>99.8</v>
       </c>
       <c r="C12">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="13">
@@ -1311,7 +1311,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="14">
@@ -1324,7 +1324,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="15">
@@ -1337,7 +1337,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
     <row r="16">
@@ -1350,7 +1350,7 @@
         <v>100</v>
       </c>
       <c r="C16">
-        <v>808</v>
+        <v>883</v>
       </c>
     </row>
   </sheetData>
@@ -1387,10 +1387,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>191</v>
+        <v>227</v>
       </c>
       <c r="C2">
-        <v>23.6</v>
+        <v>25.7</v>
       </c>
     </row>
     <row r="3">
@@ -1400,10 +1400,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="C3">
-        <v>12.9</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="4">
@@ -1413,10 +1413,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="C4">
-        <v>12.7</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="5">
@@ -1426,10 +1426,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="C5">
-        <v>11.4</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="6">
@@ -1439,10 +1439,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="C6">
-        <v>8.699999999999999</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="7">
@@ -1452,10 +1452,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C7">
-        <v>2.1</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="8">
@@ -1465,10 +1465,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C8">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="9">
@@ -1478,10 +1478,10 @@
         </is>
       </c>
       <c r="B9">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="10">
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -1507,7 +1507,7 @@
         <v>7</v>
       </c>
       <c r="C11">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="12">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1578,7 +1578,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1642,13 +1642,13 @@
         </is>
       </c>
       <c r="B7">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7">
-        <v>5.3</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="8">
@@ -1658,13 +1658,13 @@
         </is>
       </c>
       <c r="B8">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="9">
@@ -1674,13 +1674,13 @@
         </is>
       </c>
       <c r="B9">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="10">
@@ -1690,13 +1690,13 @@
         </is>
       </c>
       <c r="B10">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C10">
         <v>5</v>
       </c>
       <c r="D10">
-        <v>11.4</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="11">
@@ -1706,7 +1706,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1722,13 +1722,13 @@
         </is>
       </c>
       <c r="B12">
-        <v>302</v>
+        <v>344</v>
       </c>
       <c r="C12">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D12">
-        <v>11.6</v>
+        <v>11.3</v>
       </c>
     </row>
   </sheetData>
@@ -1770,13 +1770,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="C2">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D2">
-        <v>45.6</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="3">
@@ -1786,13 +1786,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C3">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D3">
-        <v>17.2</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="4">
@@ -1850,13 +1850,13 @@
         </is>
       </c>
       <c r="B7">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7">
-        <v>31.6</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="8">
@@ -1866,13 +1866,13 @@
         </is>
       </c>
       <c r="B8">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C8">
         <v>10</v>
       </c>
       <c r="D8">
-        <v>34.5</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="9">
@@ -1882,13 +1882,13 @@
         </is>
       </c>
       <c r="B9">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C9">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D9">
-        <v>23.4</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -1898,13 +1898,13 @@
         </is>
       </c>
       <c r="B10">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C10">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D10">
-        <v>43.2</v>
+        <v>40.8</v>
       </c>
     </row>
     <row r="11">
@@ -1914,13 +1914,13 @@
         </is>
       </c>
       <c r="B11">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C11">
         <v>18</v>
       </c>
       <c r="D11">
-        <v>22.8</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="12">
@@ -1930,13 +1930,13 @@
         </is>
       </c>
       <c r="B12">
-        <v>302</v>
+        <v>344</v>
       </c>
       <c r="C12">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="D12">
-        <v>30.8</v>
+        <v>30.5</v>
       </c>
     </row>
   </sheetData>
@@ -1973,10 +1973,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>355</v>
+        <v>420</v>
       </c>
       <c r="C2">
-        <v>97.5</v>
+        <v>97.7</v>
       </c>
     </row>
     <row r="3">
@@ -1986,7 +1986,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3">
         <v>1.9</v>
@@ -2039,10 +2039,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="C2">
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="3">
@@ -2052,10 +2052,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>608</v>
+        <v>672</v>
       </c>
       <c r="C3">
-        <v>75.2</v>
+        <v>76.09999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -2065,10 +2065,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>164</v>
+        <v>189</v>
       </c>
       <c r="C4">
-        <v>20.3</v>
+        <v>21.4</v>
       </c>
     </row>
   </sheetData>
@@ -2118,10 +2118,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>367</v>
+        <v>392</v>
       </c>
       <c r="C3">
-        <v>45.4</v>
+        <v>44.4</v>
       </c>
     </row>
     <row r="4">
@@ -2131,10 +2131,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>439</v>
+        <v>489</v>
       </c>
       <c r="C4">
-        <v>54.3</v>
+        <v>55.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização de dados — 01/07/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -406,48 +406,48 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Uniflor</t>
+          <t>Nova Esperanca</t>
         </is>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>71</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E2">
-        <v>237.4</v>
+        <v>261.6</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Nova Esperanca</t>
+          <t>Uniflor</t>
         </is>
       </c>
       <c r="B3">
-        <v>63</v>
+        <v>5</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>232.1</v>
+        <v>237.4</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -456,13 +456,13 @@
         <v>0</v>
       </c>
       <c r="H3">
-        <v>6.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Atalaia</t>
+          <t>Nossa Senhora Das Gracas</t>
         </is>
       </c>
       <c r="B4">
@@ -472,10 +472,10 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E4">
-        <v>173</v>
+        <v>190.8</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -484,26 +484,26 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Nossa Senhora Das Gracas</t>
+          <t>Atalaia</t>
         </is>
       </c>
       <c r="B5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>163.5</v>
+        <v>173</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -512,26 +512,26 @@
         <v>0</v>
       </c>
       <c r="H5">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Santo Inacio</t>
+          <t>Ourizona</t>
         </is>
       </c>
       <c r="B6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6">
-        <v>154.7</v>
+        <v>156.6</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -546,29 +546,29 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Itaguaje</t>
+          <t>Santo Inacio</t>
         </is>
       </c>
       <c r="B7">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7">
-        <v>154.5</v>
+        <v>154.7</v>
       </c>
       <c r="F7">
-        <v>22.1</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>14.3</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>14.3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
@@ -578,81 +578,81 @@
         </is>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8">
         <v>3</v>
       </c>
       <c r="E8">
-        <v>135.4</v>
+        <v>154.7</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>19.3</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>12.5</v>
       </c>
       <c r="H8">
-        <v>42.9</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Maringa</t>
+          <t>Itaguaje</t>
         </is>
       </c>
       <c r="B9">
-        <v>556</v>
+        <v>7</v>
       </c>
       <c r="C9">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="D9">
-        <v>159</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>129.4</v>
+        <v>154.5</v>
       </c>
       <c r="F9">
-        <v>9.1</v>
+        <v>22.1</v>
       </c>
       <c r="G9">
-        <v>7</v>
+        <v>14.3</v>
       </c>
       <c r="H9">
-        <v>28.6</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ourizona</t>
+          <t>Maringa</t>
         </is>
       </c>
       <c r="B10">
-        <v>4</v>
+        <v>624</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>177</v>
       </c>
       <c r="E10">
-        <v>125.3</v>
+        <v>145.2</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>11.4</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>7.9</v>
       </c>
       <c r="H10">
-        <v>25</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="11">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>2</v>
       </c>
       <c r="E11">
-        <v>111.5</v>
+        <v>124.4</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -680,63 +680,63 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>7.7</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Florai</t>
+          <t>Marialva</t>
         </is>
       </c>
       <c r="B12">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E12">
-        <v>83.2</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="H12">
-        <v>25</v>
+        <v>44.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Marialva</t>
+          <t>Florai</t>
         </is>
       </c>
       <c r="B13">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="C13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D13">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E13">
-        <v>76</v>
+        <v>83.2</v>
       </c>
       <c r="F13">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>5.9</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>47.1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14">
@@ -770,57 +770,57 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Itambe</t>
+          <t>Sarandi</t>
         </is>
       </c>
       <c r="B15">
-        <v>4</v>
+        <v>87</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="E15">
-        <v>64.2</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>4.7</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="H15">
-        <v>25</v>
+        <v>39.1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sarandi</t>
+          <t>Itambe</t>
         </is>
       </c>
       <c r="B16">
-        <v>79</v>
+        <v>4</v>
       </c>
       <c r="C16">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E16">
-        <v>61.7</v>
+        <v>64.2</v>
       </c>
       <c r="F16">
-        <v>3.9</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>6.3</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>41.8</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17">
@@ -854,20 +854,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Lobato</t>
+          <t>Floresta</t>
         </is>
       </c>
       <c r="B18">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C18">
         <v>0</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18">
-        <v>42.5</v>
+        <v>52.1</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -876,26 +876,26 @@
         <v>0</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mandaguacu</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="B19">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C19">
         <v>0</v>
       </c>
       <c r="D19">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E19">
-        <v>40.6</v>
+        <v>42.6</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -904,26 +904,26 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>35.7</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Astorga</t>
+          <t>Lobato</t>
         </is>
       </c>
       <c r="B20">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
       <c r="D20">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E20">
-        <v>38.2</v>
+        <v>42.5</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -932,73 +932,73 @@
         <v>0</v>
       </c>
       <c r="H20">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Paicandu</t>
+          <t>Mandaguacu</t>
         </is>
       </c>
       <c r="B21">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E21">
-        <v>37</v>
+        <v>40.6</v>
       </c>
       <c r="F21">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="G21">
-        <v>5.6</v>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>55.6</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Floresta</t>
+          <t>Paicandu</t>
         </is>
       </c>
       <c r="B22">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E22">
-        <v>34.7</v>
+        <v>37</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>5.6</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>55.6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Astorga</t>
         </is>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -1007,7 +1007,7 @@
         <v>3</v>
       </c>
       <c r="E23">
-        <v>34.1</v>
+        <v>34.3</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -1016,7 +1016,7 @@
         <v>0</v>
       </c>
       <c r="H23">
-        <v>75</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="24">
@@ -1050,20 +1050,20 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mandaguari</t>
+          <t>Presidente Castelo Branco</t>
         </is>
       </c>
       <c r="B25">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E25">
-        <v>20.9</v>
+        <v>23.2</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1072,26 +1072,26 @@
         <v>0</v>
       </c>
       <c r="H25">
-        <v>75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Iguaracu</t>
+          <t>Mandaguari</t>
         </is>
       </c>
       <c r="B26">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C26">
         <v>0</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E26">
-        <v>17.6</v>
+        <v>20.9</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -1100,13 +1100,13 @@
         <v>0</v>
       </c>
       <c r="H26">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Doutor Camargo</t>
+          <t>Iguaracu</t>
         </is>
       </c>
       <c r="B27">
@@ -1116,18 +1116,46 @@
         <v>0</v>
       </c>
       <c r="D27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27">
+        <v>17.6</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Doutor Camargo</t>
+        </is>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
         <v>15.3</v>
       </c>
-      <c r="F27">
-        <v>0</v>
-      </c>
-      <c r="G27">
-        <v>0</v>
-      </c>
-      <c r="H27">
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
         <v>0</v>
       </c>
     </row>
@@ -1165,10 +1193,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>56.4</v>
+        <v>58.7</v>
       </c>
       <c r="C2">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="3">
@@ -1178,36 +1206,36 @@
         </is>
       </c>
       <c r="B3">
-        <v>56.5</v>
+        <v>58.8</v>
       </c>
       <c r="C3">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cardiopatia</t>
+          <t>Imunodepressão</t>
         </is>
       </c>
       <c r="B4">
-        <v>56.6</v>
+        <v>58.8</v>
       </c>
       <c r="C4">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Imunodepressão</t>
+          <t>Cardiopatia</t>
         </is>
       </c>
       <c r="B5">
-        <v>56.6</v>
+        <v>58.9</v>
       </c>
       <c r="C5">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="6">
@@ -1217,10 +1245,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>61.5</v>
+        <v>63</v>
       </c>
       <c r="C6">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="7">
@@ -1230,10 +1258,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>77.3</v>
+        <v>80.8</v>
       </c>
       <c r="C7">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="8">
@@ -1243,10 +1271,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>90.09999999999999</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="C8">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="9">
@@ -1256,10 +1284,10 @@
         </is>
       </c>
       <c r="B9">
-        <v>94.5</v>
+        <v>95.5</v>
       </c>
       <c r="C9">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="10">
@@ -1272,7 +1300,7 @@
         <v>97.5</v>
       </c>
       <c r="C10">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="11">
@@ -1282,10 +1310,10 @@
         </is>
       </c>
       <c r="B11">
-        <v>99.7</v>
+        <v>99.5</v>
       </c>
       <c r="C11">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="12">
@@ -1298,7 +1326,7 @@
         <v>99.8</v>
       </c>
       <c r="C12">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="13">
@@ -1311,7 +1339,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="14">
@@ -1324,7 +1352,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="15">
@@ -1337,7 +1365,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
     <row r="16">
@@ -1350,7 +1378,7 @@
         <v>100</v>
       </c>
       <c r="C16">
-        <v>883</v>
+        <v>985</v>
       </c>
     </row>
   </sheetData>
@@ -1387,10 +1415,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>227</v>
+        <v>271</v>
       </c>
       <c r="C2">
-        <v>25.7</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="3">
@@ -1400,10 +1428,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="C3">
-        <v>13.3</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="4">
@@ -1413,10 +1441,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="C4">
-        <v>13.3</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="5">
@@ -1426,10 +1454,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="C5">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="6">
@@ -1439,10 +1467,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="C6">
-        <v>9.9</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="7">
@@ -1452,10 +1480,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C7">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="8">
@@ -1465,10 +1493,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C8">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="9">
@@ -1478,7 +1506,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C9">
         <v>2.2</v>
@@ -1494,7 +1522,7 @@
         <v>9</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="11">
@@ -1504,10 +1532,10 @@
         </is>
       </c>
       <c r="B11">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C11">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="12">
@@ -1562,13 +1590,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1578,7 +1606,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1626,7 +1654,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1642,13 +1670,13 @@
         </is>
       </c>
       <c r="B7">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7">
-        <v>4.8</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="8">
@@ -1658,13 +1686,13 @@
         </is>
       </c>
       <c r="B8">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="9">
@@ -1674,7 +1702,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1690,13 +1718,13 @@
         </is>
       </c>
       <c r="B10">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D10">
-        <v>10.2</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="11">
@@ -1706,7 +1734,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1722,13 +1750,13 @@
         </is>
       </c>
       <c r="B12">
-        <v>344</v>
+        <v>411</v>
       </c>
       <c r="C12">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="D12">
-        <v>11.3</v>
+        <v>11.9</v>
       </c>
     </row>
   </sheetData>
@@ -1770,13 +1798,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="C2">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D2">
-        <v>45.5</v>
+        <v>43.9</v>
       </c>
     </row>
     <row r="3">
@@ -1786,13 +1814,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="C3">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D3">
-        <v>17.9</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="4">
@@ -1805,10 +1833,10 @@
         <v>21</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4">
-        <v>28.6</v>
+        <v>23.8</v>
       </c>
     </row>
     <row r="5">
@@ -1834,13 +1862,13 @@
         </is>
       </c>
       <c r="B6">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6">
-        <v>30.8</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="7">
@@ -1850,13 +1878,13 @@
         </is>
       </c>
       <c r="B7">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D7">
-        <v>33.3</v>
+        <v>30.8</v>
       </c>
     </row>
     <row r="8">
@@ -1866,13 +1894,13 @@
         </is>
       </c>
       <c r="B8">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C8">
         <v>10</v>
       </c>
       <c r="D8">
-        <v>31.2</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="9">
@@ -1882,13 +1910,13 @@
         </is>
       </c>
       <c r="B9">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C9">
         <v>17</v>
       </c>
       <c r="D9">
-        <v>25</v>
+        <v>25.8</v>
       </c>
     </row>
     <row r="10">
@@ -1898,13 +1926,13 @@
         </is>
       </c>
       <c r="B10">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C10">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D10">
-        <v>40.8</v>
+        <v>39.6</v>
       </c>
     </row>
     <row r="11">
@@ -1914,13 +1942,13 @@
         </is>
       </c>
       <c r="B11">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C11">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D11">
-        <v>21.4</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="12">
@@ -1930,13 +1958,13 @@
         </is>
       </c>
       <c r="B12">
-        <v>344</v>
+        <v>411</v>
       </c>
       <c r="C12">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="D12">
-        <v>30.5</v>
+        <v>28.7</v>
       </c>
     </row>
   </sheetData>
@@ -1973,10 +2001,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>420</v>
+        <v>492</v>
       </c>
       <c r="C2">
-        <v>97.7</v>
+        <v>96.5</v>
       </c>
     </row>
     <row r="3">
@@ -1986,10 +2014,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C3">
-        <v>1.9</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="4">
@@ -2002,7 +2030,7 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>
@@ -2039,7 +2067,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C2">
         <v>2.5</v>
@@ -2052,10 +2080,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>672</v>
+        <v>745</v>
       </c>
       <c r="C3">
-        <v>76.09999999999999</v>
+        <v>75.59999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -2065,10 +2093,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>189</v>
+        <v>215</v>
       </c>
       <c r="C4">
-        <v>21.4</v>
+        <v>21.8</v>
       </c>
     </row>
   </sheetData>
@@ -2118,10 +2146,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>392</v>
+        <v>418</v>
       </c>
       <c r="C3">
-        <v>44.4</v>
+        <v>42.4</v>
       </c>
     </row>
     <row r="4">
@@ -2131,10 +2159,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>489</v>
+        <v>565</v>
       </c>
       <c r="C4">
-        <v>55.4</v>
+        <v>57.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização de dados — 16/07/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -410,25 +410,25 @@
         </is>
       </c>
       <c r="B2">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="C2">
         <v>2</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>261.6</v>
+        <v>320.5</v>
       </c>
       <c r="F2">
         <v>7.4</v>
       </c>
       <c r="G2">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="H2">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="3">
@@ -462,20 +462,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nossa Senhora Das Gracas</t>
+          <t>Atalaia</t>
         </is>
       </c>
       <c r="B4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>190.8</v>
+        <v>197.7</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -484,54 +484,54 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>42.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Atalaia</t>
+          <t>Sao Jorge Do Ivai</t>
         </is>
       </c>
       <c r="B5">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E5">
-        <v>173</v>
+        <v>193.4</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>19.3</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ourizona</t>
+          <t>Nossa Senhora Das Gracas</t>
         </is>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E6">
-        <v>156.6</v>
+        <v>190.8</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -540,119 +540,119 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>20</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Santo Inacio</t>
+          <t>Maringa</t>
         </is>
       </c>
       <c r="B7">
-        <v>10</v>
+        <v>708</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>191</v>
       </c>
       <c r="E7">
-        <v>154.7</v>
+        <v>164.8</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>14.9</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H7">
-        <v>20</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sao Jorge Do Ivai</t>
+          <t>Ourizona</t>
         </is>
       </c>
       <c r="B8">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
         <v>1</v>
       </c>
-      <c r="D8">
-        <v>3</v>
-      </c>
       <c r="E8">
-        <v>154.7</v>
+        <v>156.6</v>
       </c>
       <c r="F8">
-        <v>19.3</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>37.5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Itaguaje</t>
+          <t>Santo Inacio</t>
         </is>
       </c>
       <c r="B9">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9">
-        <v>154.5</v>
+        <v>154.7</v>
       </c>
       <c r="F9">
-        <v>22.1</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>14.3</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>14.3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Maringa</t>
+          <t>Itaguaje</t>
         </is>
       </c>
       <c r="B10">
-        <v>624</v>
+        <v>7</v>
       </c>
       <c r="C10">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="D10">
-        <v>177</v>
+        <v>1</v>
       </c>
       <c r="E10">
-        <v>145.2</v>
+        <v>154.5</v>
       </c>
       <c r="F10">
-        <v>11.4</v>
+        <v>22.1</v>
       </c>
       <c r="G10">
-        <v>7.9</v>
+        <v>14.3</v>
       </c>
       <c r="H10">
-        <v>28.4</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="11">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>2</v>
       </c>
       <c r="E11">
-        <v>124.4</v>
+        <v>150.1</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -680,54 +680,54 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>6.9</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Marialva</t>
+          <t>Florai</t>
         </is>
       </c>
       <c r="B12">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D12">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E12">
-        <v>96.09999999999999</v>
+        <v>124.9</v>
       </c>
       <c r="F12">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>44.2</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Florai</t>
+          <t>Itambe</t>
         </is>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C13">
         <v>0</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13">
-        <v>83.2</v>
+        <v>112.4</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -736,91 +736,91 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>25</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Paranacity</t>
+          <t>Marialva</t>
         </is>
       </c>
       <c r="B14">
-        <v>7</v>
+        <v>49</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D14">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="E14">
-        <v>73.3</v>
+        <v>109.5</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>4.1</v>
       </c>
       <c r="H14">
-        <v>14.3</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sarandi</t>
+          <t>Paranacity</t>
         </is>
       </c>
       <c r="B15">
-        <v>87</v>
+        <v>9</v>
       </c>
       <c r="C15">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D15">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E15">
-        <v>67.90000000000001</v>
+        <v>94.3</v>
       </c>
       <c r="F15">
-        <v>4.7</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>6.9</v>
+        <v>0</v>
       </c>
       <c r="H15">
-        <v>39.1</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Itambe</t>
+          <t>Sarandi</t>
         </is>
       </c>
       <c r="B16">
-        <v>4</v>
+        <v>95</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D16">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E16">
-        <v>64.2</v>
+        <v>74.2</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="H16">
-        <v>25</v>
+        <v>38.9</v>
       </c>
     </row>
     <row r="17">
@@ -882,20 +882,20 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Presidente Castelo Branco</t>
         </is>
       </c>
       <c r="B19">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C19">
         <v>0</v>
       </c>
       <c r="D19">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E19">
-        <v>42.6</v>
+        <v>46.5</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -904,26 +904,26 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Lobato</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E20">
-        <v>42.5</v>
+        <v>42.6</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -932,26 +932,26 @@
         <v>0</v>
       </c>
       <c r="H20">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Mandaguacu</t>
+          <t>Lobato</t>
         </is>
       </c>
       <c r="B21">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>40.6</v>
+        <v>42.5</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -960,7 +960,7 @@
         <v>0</v>
       </c>
       <c r="H21">
-        <v>35.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -970,44 +970,44 @@
         </is>
       </c>
       <c r="B22">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C22">
         <v>1</v>
       </c>
       <c r="D22">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E22">
-        <v>37</v>
+        <v>41.1</v>
       </c>
       <c r="F22">
         <v>2.1</v>
       </c>
       <c r="G22">
-        <v>5.6</v>
+        <v>5</v>
       </c>
       <c r="H22">
-        <v>55.6</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Astorga</t>
+          <t>Mandaguacu</t>
         </is>
       </c>
       <c r="B23">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C23">
         <v>0</v>
       </c>
       <c r="D23">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E23">
-        <v>34.3</v>
+        <v>40.6</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -1016,26 +1016,26 @@
         <v>0</v>
       </c>
       <c r="H23">
-        <v>33.3</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Munhoz De Melo</t>
+          <t>Astorga</t>
         </is>
       </c>
       <c r="B24">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C24">
         <v>0</v>
       </c>
       <c r="D24">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E24">
-        <v>24.6</v>
+        <v>38.2</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -1044,26 +1044,26 @@
         <v>0</v>
       </c>
       <c r="H24">
-        <v>100</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Presidente Castelo Branco</t>
+          <t>Mandaguari</t>
         </is>
       </c>
       <c r="B25">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E25">
-        <v>23.2</v>
+        <v>26.1</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1072,26 +1072,26 @@
         <v>0</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mandaguari</t>
+          <t>Munhoz De Melo</t>
         </is>
       </c>
       <c r="B26">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C26">
         <v>0</v>
       </c>
       <c r="D26">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E26">
-        <v>20.9</v>
+        <v>24.6</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -1100,7 +1100,7 @@
         <v>0</v>
       </c>
       <c r="H26">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27">
@@ -1193,10 +1193,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>58.7</v>
+        <v>58.8</v>
       </c>
       <c r="C2">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="3">
@@ -1206,36 +1206,36 @@
         </is>
       </c>
       <c r="B3">
-        <v>58.8</v>
+        <v>58.9</v>
       </c>
       <c r="C3">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Imunodepressão</t>
+          <t>Cardiopatia</t>
         </is>
       </c>
       <c r="B4">
-        <v>58.8</v>
+        <v>59</v>
       </c>
       <c r="C4">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cardiopatia</t>
+          <t>Imunodepressão</t>
         </is>
       </c>
       <c r="B5">
-        <v>58.9</v>
+        <v>59</v>
       </c>
       <c r="C5">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="6">
@@ -1245,10 +1245,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C6">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="7">
@@ -1258,10 +1258,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>80.8</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="C7">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="8">
@@ -1271,10 +1271,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>89.90000000000001</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="C8">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="9">
@@ -1284,10 +1284,10 @@
         </is>
       </c>
       <c r="B9">
-        <v>95.5</v>
+        <v>96</v>
       </c>
       <c r="C9">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="10">
@@ -1297,10 +1297,10 @@
         </is>
       </c>
       <c r="B10">
-        <v>97.5</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="C10">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="11">
@@ -1310,10 +1310,10 @@
         </is>
       </c>
       <c r="B11">
-        <v>99.5</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="C11">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="12">
@@ -1326,7 +1326,7 @@
         <v>99.8</v>
       </c>
       <c r="C12">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="13">
@@ -1339,7 +1339,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="14">
@@ -1352,7 +1352,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="15">
@@ -1365,7 +1365,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="16">
@@ -1378,7 +1378,7 @@
         <v>100</v>
       </c>
       <c r="C16">
-        <v>985</v>
+        <v>1121</v>
       </c>
     </row>
   </sheetData>
@@ -1415,10 +1415,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>271</v>
+        <v>322</v>
       </c>
       <c r="C2">
-        <v>27.5</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="3">
@@ -1428,10 +1428,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>133</v>
+        <v>162</v>
       </c>
       <c r="C3">
-        <v>13.5</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="4">
@@ -1441,10 +1441,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="C4">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="5">
@@ -1454,10 +1454,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="C5">
-        <v>11.7</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="6">
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="C6">
         <v>10.8</v>
@@ -1480,36 +1480,36 @@
         </is>
       </c>
       <c r="B7">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C7">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Imunodepressão</t>
+          <t>Obesidade</t>
         </is>
       </c>
       <c r="B8">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C8">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Obesidade</t>
+          <t>Imunodepressão</t>
         </is>
       </c>
       <c r="B9">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C9">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="10">
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C10">
         <v>0.9</v>
@@ -1532,7 +1532,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C11">
         <v>0.6</v>
@@ -1590,13 +1590,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="3">
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1622,7 +1622,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1638,13 +1638,13 @@
         </is>
       </c>
       <c r="B5">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5">
-        <v>14.3</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="6">
@@ -1670,13 +1670,13 @@
         </is>
       </c>
       <c r="B7">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
       <c r="D7">
-        <v>7.7</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="8">
@@ -1686,13 +1686,13 @@
         </is>
       </c>
       <c r="B8">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="9">
@@ -1702,13 +1702,13 @@
         </is>
       </c>
       <c r="B9">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="10">
@@ -1718,13 +1718,13 @@
         </is>
       </c>
       <c r="B10">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D10">
-        <v>13.2</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="11">
@@ -1734,7 +1734,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1750,13 +1750,13 @@
         </is>
       </c>
       <c r="B12">
-        <v>411</v>
+        <v>481</v>
       </c>
       <c r="C12">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="D12">
-        <v>11.9</v>
+        <v>13.3</v>
       </c>
     </row>
   </sheetData>
@@ -1798,13 +1798,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="C2">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D2">
-        <v>43.9</v>
+        <v>45.8</v>
       </c>
     </row>
     <row r="3">
@@ -1814,13 +1814,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="C3">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D3">
-        <v>20.5</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="4">
@@ -1830,13 +1830,13 @@
         </is>
       </c>
       <c r="B4">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C4">
         <v>5</v>
       </c>
       <c r="D4">
-        <v>23.8</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="5">
@@ -1846,13 +1846,13 @@
         </is>
       </c>
       <c r="B5">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
       <c r="D5">
-        <v>28.6</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="6">
@@ -1865,10 +1865,10 @@
         <v>15</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D6">
-        <v>33.3</v>
+        <v>26.7</v>
       </c>
     </row>
     <row r="7">
@@ -1878,13 +1878,13 @@
         </is>
       </c>
       <c r="B7">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D7">
-        <v>30.8</v>
+        <v>32.1</v>
       </c>
     </row>
     <row r="8">
@@ -1894,13 +1894,13 @@
         </is>
       </c>
       <c r="B8">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C8">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D8">
-        <v>28.6</v>
+        <v>29.7</v>
       </c>
     </row>
     <row r="9">
@@ -1910,13 +1910,13 @@
         </is>
       </c>
       <c r="B9">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="C9">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D9">
-        <v>25.8</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -1926,13 +1926,13 @@
         </is>
       </c>
       <c r="B10">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C10">
         <v>21</v>
       </c>
       <c r="D10">
-        <v>39.6</v>
+        <v>35.6</v>
       </c>
     </row>
     <row r="11">
@@ -1942,13 +1942,13 @@
         </is>
       </c>
       <c r="B11">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C11">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D11">
-        <v>19.5</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="12">
@@ -1958,13 +1958,13 @@
         </is>
       </c>
       <c r="B12">
-        <v>411</v>
+        <v>481</v>
       </c>
       <c r="C12">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="D12">
-        <v>28.7</v>
+        <v>27.2</v>
       </c>
     </row>
   </sheetData>
@@ -2001,10 +2001,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>492</v>
+        <v>566</v>
       </c>
       <c r="C2">
-        <v>96.5</v>
+        <v>94.59999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -2014,10 +2014,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3">
-        <v>3.1</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="4">
@@ -2027,10 +2027,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C4">
-        <v>0.4</v>
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>
@@ -2067,10 +2067,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C2">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="3">
@@ -2080,10 +2080,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>745</v>
+        <v>841</v>
       </c>
       <c r="C3">
-        <v>75.59999999999999</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4">
@@ -2093,10 +2093,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>215</v>
+        <v>251</v>
       </c>
       <c r="C4">
-        <v>21.8</v>
+        <v>22.4</v>
       </c>
     </row>
   </sheetData>
@@ -2146,10 +2146,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>418</v>
+        <v>465</v>
       </c>
       <c r="C3">
-        <v>42.4</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="4">
@@ -2159,10 +2159,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>565</v>
+        <v>654</v>
       </c>
       <c r="C4">
-        <v>57.4</v>
+        <v>58.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização de dados — 17/08/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -358,7 +358,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -410,25 +410,25 @@
         </is>
       </c>
       <c r="B2">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D2">
         <v>5</v>
       </c>
       <c r="E2">
-        <v>320.5</v>
+        <v>361.1</v>
       </c>
       <c r="F2">
-        <v>7.4</v>
+        <v>18.4</v>
       </c>
       <c r="G2">
-        <v>2.3</v>
+        <v>5.1</v>
       </c>
       <c r="H2">
-        <v>5.7</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="3">
@@ -438,22 +438,22 @@
         </is>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3">
-        <v>237.4</v>
+        <v>284.9</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>47.5</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>16.7</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -466,7 +466,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -475,7 +475,7 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>197.7</v>
+        <v>222.4</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -490,7 +490,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sao Jorge Do Ivai</t>
+          <t>Itaguaje</t>
         </is>
       </c>
       <c r="B5">
@@ -500,25 +500,25 @@
         <v>1</v>
       </c>
       <c r="D5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E5">
-        <v>193.4</v>
+        <v>220.8</v>
       </c>
       <c r="F5">
-        <v>19.3</v>
+        <v>22.1</v>
       </c>
       <c r="G5">
         <v>10</v>
       </c>
       <c r="H5">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nossa Senhora Das Gracas</t>
+          <t>Ourizona</t>
         </is>
       </c>
       <c r="B6">
@@ -531,7 +531,7 @@
         <v>3</v>
       </c>
       <c r="E6">
-        <v>190.8</v>
+        <v>219.2</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -546,113 +546,113 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Maringa</t>
+          <t>Nossa Senhora Das Gracas</t>
         </is>
       </c>
       <c r="B7">
-        <v>708</v>
+        <v>8</v>
       </c>
       <c r="C7">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>191</v>
+        <v>3</v>
       </c>
       <c r="E7">
-        <v>164.8</v>
+        <v>218</v>
       </c>
       <c r="F7">
-        <v>14.9</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>27</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ourizona</t>
+          <t>Sao Jorge Do Ivai</t>
         </is>
       </c>
       <c r="B8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8">
-        <v>156.6</v>
+        <v>212.8</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>19.3</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>9.1</v>
       </c>
       <c r="H8">
-        <v>20</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Santo Inacio</t>
+          <t>Maringa</t>
         </is>
       </c>
       <c r="B9">
-        <v>10</v>
+        <v>829</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>235</v>
       </c>
       <c r="E9">
-        <v>154.7</v>
+        <v>192.9</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>18.9</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H9">
-        <v>20</v>
+        <v>28.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Itaguaje</t>
+          <t>Santo Inacio</t>
         </is>
       </c>
       <c r="B10">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10">
-        <v>154.5</v>
+        <v>185.7</v>
       </c>
       <c r="F10">
-        <v>22.1</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>14.3</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>14.3</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="11">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -671,7 +671,7 @@
         <v>2</v>
       </c>
       <c r="E11">
-        <v>150.1</v>
+        <v>175.9</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -680,26 +680,26 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>5.7</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Florai</t>
+          <t>Itambe</t>
         </is>
       </c>
       <c r="B12">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C12">
         <v>0</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12">
-        <v>124.9</v>
+        <v>160.6</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -708,26 +708,26 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>16.7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Itambe</t>
+          <t>Florai</t>
         </is>
       </c>
       <c r="B13">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C13">
         <v>0</v>
       </c>
       <c r="D13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13">
-        <v>112.4</v>
+        <v>124.9</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -736,7 +736,7 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>28.6</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="14">
@@ -746,44 +746,44 @@
         </is>
       </c>
       <c r="B14">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C14">
         <v>2</v>
       </c>
       <c r="D14">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E14">
-        <v>109.5</v>
+        <v>120.7</v>
       </c>
       <c r="F14">
         <v>4.5</v>
       </c>
       <c r="G14">
-        <v>4.1</v>
+        <v>3.7</v>
       </c>
       <c r="H14">
-        <v>49</v>
+        <v>46.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Paranacity</t>
+          <t>Santa Ines</t>
         </is>
       </c>
       <c r="B15">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C15">
         <v>0</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15">
-        <v>94.3</v>
+        <v>114.6</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -792,110 +792,110 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>11.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sarandi</t>
+          <t>Paranacity</t>
         </is>
       </c>
       <c r="B16">
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="C16">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E16">
-        <v>74.2</v>
+        <v>104.7</v>
       </c>
       <c r="F16">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>38.9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Santa Ines</t>
+          <t>Sarandi</t>
         </is>
       </c>
       <c r="B17">
-        <v>1</v>
+        <v>108</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D17">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="E17">
-        <v>57.3</v>
+        <v>84.3</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>38.9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Floresta</t>
+          <t>Astorga</t>
         </is>
       </c>
       <c r="B18">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E18">
-        <v>52.1</v>
+        <v>53.4</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>7.1</v>
       </c>
       <c r="H18">
-        <v>16.7</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Presidente Castelo Branco</t>
+          <t>Floresta</t>
         </is>
       </c>
       <c r="B19">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C19">
         <v>0</v>
       </c>
       <c r="D19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19">
-        <v>46.5</v>
+        <v>52.1</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -904,26 +904,26 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>0</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Munhoz De Melo</t>
         </is>
       </c>
       <c r="B20">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
       <c r="D20">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E20">
-        <v>42.6</v>
+        <v>49.3</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -932,26 +932,26 @@
         <v>0</v>
       </c>
       <c r="H20">
-        <v>80</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Lobato</t>
+          <t>Mandaguacu</t>
         </is>
       </c>
       <c r="B21">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E21">
-        <v>42.5</v>
+        <v>49.2</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -960,82 +960,82 @@
         <v>0</v>
       </c>
       <c r="H21">
-        <v>0</v>
+        <v>41.2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Paicandu</t>
+          <t>Presidente Castelo Branco</t>
         </is>
       </c>
       <c r="B22">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E22">
-        <v>41.1</v>
+        <v>46.5</v>
       </c>
       <c r="F22">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>55</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Mandaguacu</t>
+          <t>Paicandu</t>
         </is>
       </c>
       <c r="B23">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="E23">
-        <v>40.6</v>
+        <v>45.2</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="H23">
-        <v>35.7</v>
+        <v>59.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Astorga</t>
+          <t>Santa Fe</t>
         </is>
       </c>
       <c r="B24">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C24">
         <v>0</v>
       </c>
       <c r="D24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E24">
-        <v>38.2</v>
+        <v>42.6</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -1044,26 +1044,26 @@
         <v>0</v>
       </c>
       <c r="H24">
-        <v>30</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mandaguari</t>
+          <t>Lobato</t>
         </is>
       </c>
       <c r="B25">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E25">
-        <v>26.1</v>
+        <v>42.5</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1072,13 +1072,13 @@
         <v>0</v>
       </c>
       <c r="H25">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Munhoz De Melo</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="B26">
@@ -1091,7 +1091,7 @@
         <v>1</v>
       </c>
       <c r="E26">
-        <v>24.6</v>
+        <v>36.9</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="B27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -1119,7 +1119,7 @@
         <v>1</v>
       </c>
       <c r="E27">
-        <v>17.6</v>
+        <v>35.1</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -1128,35 +1128,63 @@
         <v>0</v>
       </c>
       <c r="H27">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>Mandaguari</t>
+        </is>
+      </c>
+      <c r="B28">
+        <v>13</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>10</v>
+      </c>
+      <c r="E28">
+        <v>33.9</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>76.90000000000001</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>Doutor Camargo</t>
         </is>
       </c>
-      <c r="B28">
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29">
+        <v>0</v>
+      </c>
+      <c r="D29">
         <v>1</v>
       </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
-      <c r="D28">
-        <v>0</v>
-      </c>
-      <c r="E28">
-        <v>15.3</v>
-      </c>
-      <c r="F28">
-        <v>0</v>
-      </c>
-      <c r="G28">
-        <v>0</v>
-      </c>
-      <c r="H28">
-        <v>0</v>
+      <c r="E29">
+        <v>30.7</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1193,10 +1221,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>58.8</v>
+        <v>59.9</v>
       </c>
       <c r="C2">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="3">
@@ -1206,10 +1234,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>58.9</v>
+        <v>60.4</v>
       </c>
       <c r="C3">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="4">
@@ -1219,10 +1247,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>59</v>
+        <v>60.5</v>
       </c>
       <c r="C4">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="5">
@@ -1232,10 +1260,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>59</v>
+        <v>60.5</v>
       </c>
       <c r="C5">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="6">
@@ -1245,10 +1273,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>68</v>
+        <v>79.5</v>
       </c>
       <c r="C6">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="7">
@@ -1258,10 +1286,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>82.40000000000001</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="C7">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="8">
@@ -1271,49 +1299,49 @@
         </is>
       </c>
       <c r="B8">
-        <v>89.40000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="C8">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Data Internação</t>
+          <t>Antiviral</t>
         </is>
       </c>
       <c r="B9">
-        <v>96</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="C9">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Antiviral</t>
+          <t>Raça/Cor</t>
         </is>
       </c>
       <c r="B10">
-        <v>97.40000000000001</v>
+        <v>98.5</v>
       </c>
       <c r="C10">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Raça/Cor</t>
+          <t>Data Internação</t>
         </is>
       </c>
       <c r="B11">
-        <v>99.59999999999999</v>
+        <v>99</v>
       </c>
       <c r="C11">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="12">
@@ -1326,7 +1354,7 @@
         <v>99.8</v>
       </c>
       <c r="C12">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="13">
@@ -1339,7 +1367,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="14">
@@ -1352,7 +1380,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="15">
@@ -1365,7 +1393,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="16">
@@ -1378,7 +1406,7 @@
         <v>100</v>
       </c>
       <c r="C16">
-        <v>1121</v>
+        <v>1309</v>
       </c>
     </row>
   </sheetData>
@@ -1388,7 +1416,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1415,10 +1443,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>322</v>
+        <v>387</v>
       </c>
       <c r="C2">
-        <v>28.7</v>
+        <v>29.6</v>
       </c>
     </row>
     <row r="3">
@@ -1428,10 +1456,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>162</v>
+        <v>195</v>
       </c>
       <c r="C3">
-        <v>14.5</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="4">
@@ -1441,10 +1469,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="C4">
-        <v>12.5</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="5">
@@ -1454,10 +1482,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="C5">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="6">
@@ -1467,7 +1495,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>121</v>
+        <v>142</v>
       </c>
       <c r="C6">
         <v>10.8</v>
@@ -1480,10 +1508,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C7">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="8">
@@ -1493,10 +1521,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="C8">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="9">
@@ -1506,7 +1534,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C9">
         <v>2.1</v>
@@ -1522,7 +1550,7 @@
         <v>10</v>
       </c>
       <c r="C10">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="11">
@@ -1532,23 +1560,10 @@
         </is>
       </c>
       <c r="B11">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C11">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Puérpera</t>
-        </is>
-      </c>
-      <c r="B12">
-        <v>1</v>
-      </c>
-      <c r="C12">
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>
@@ -1590,13 +1605,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2">
-        <v>0.9</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3">
@@ -1606,7 +1621,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>183</v>
+        <v>220</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1622,7 +1637,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1638,13 +1653,13 @@
         </is>
       </c>
       <c r="B5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5">
-        <v>11.1</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="6">
@@ -1654,7 +1669,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1670,13 +1685,13 @@
         </is>
       </c>
       <c r="B7">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
       <c r="D7">
-        <v>7.1</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="8">
@@ -1686,13 +1701,13 @@
         </is>
       </c>
       <c r="B8">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8">
-        <v>2.7</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="9">
@@ -1702,7 +1717,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1718,13 +1733,13 @@
         </is>
       </c>
       <c r="B10">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="C10">
         <v>8</v>
       </c>
       <c r="D10">
-        <v>13.6</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="11">
@@ -1734,7 +1749,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1750,13 +1765,13 @@
         </is>
       </c>
       <c r="B12">
-        <v>481</v>
+        <v>575</v>
       </c>
       <c r="C12">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="D12">
-        <v>13.3</v>
+        <v>14.6</v>
       </c>
     </row>
   </sheetData>
@@ -1798,13 +1813,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C2">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="D2">
-        <v>45.8</v>
+        <v>44.4</v>
       </c>
     </row>
     <row r="3">
@@ -1814,13 +1829,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>183</v>
+        <v>220</v>
       </c>
       <c r="C3">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="D3">
-        <v>19.7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -1830,13 +1845,13 @@
         </is>
       </c>
       <c r="B4">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C4">
         <v>5</v>
       </c>
       <c r="D4">
-        <v>18.5</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="5">
@@ -1846,13 +1861,13 @@
         </is>
       </c>
       <c r="B5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
       <c r="D5">
-        <v>22.2</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="6">
@@ -1862,13 +1877,13 @@
         </is>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D6">
-        <v>26.7</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="7">
@@ -1878,13 +1893,13 @@
         </is>
       </c>
       <c r="B7">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D7">
-        <v>32.1</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="8">
@@ -1894,13 +1909,13 @@
         </is>
       </c>
       <c r="B8">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C8">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D8">
-        <v>29.7</v>
+        <v>34.9</v>
       </c>
     </row>
     <row r="9">
@@ -1910,13 +1925,13 @@
         </is>
       </c>
       <c r="B9">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C9">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D9">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10">
@@ -1926,13 +1941,13 @@
         </is>
       </c>
       <c r="B10">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="C10">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D10">
-        <v>35.6</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="11">
@@ -1942,13 +1957,13 @@
         </is>
       </c>
       <c r="B11">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="C11">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="D11">
-        <v>19.2</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="12">
@@ -1958,13 +1973,13 @@
         </is>
       </c>
       <c r="B12">
-        <v>481</v>
+        <v>575</v>
       </c>
       <c r="C12">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="D12">
-        <v>27.2</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -2001,10 +2016,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>566</v>
+        <v>718</v>
       </c>
       <c r="C2">
-        <v>94.59999999999999</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="3">
@@ -2014,10 +2029,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C3">
-        <v>2.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -2027,10 +2042,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="C4">
-        <v>2.5</v>
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>
@@ -2067,10 +2082,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C2">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="3">
@@ -2080,10 +2095,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>841</v>
+        <v>950</v>
       </c>
       <c r="C3">
-        <v>75</v>
+        <v>72.59999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -2093,10 +2108,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>251</v>
+        <v>327</v>
       </c>
       <c r="C4">
-        <v>22.4</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -2146,10 +2161,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>465</v>
+        <v>529</v>
       </c>
       <c r="C3">
-        <v>41.5</v>
+        <v>40.4</v>
       </c>
     </row>
     <row r="4">
@@ -2159,10 +2174,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>654</v>
+        <v>778</v>
       </c>
       <c r="C4">
-        <v>58.3</v>
+        <v>59.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização de dados — 19/08/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -18,6 +18,275 @@
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="88">
+  <si>
+    <t>municipio</t>
+  </si>
+  <si>
+    <t>casos</t>
+  </si>
+  <si>
+    <t>obitos_srag</t>
+  </si>
+  <si>
+    <t>uti</t>
+  </si>
+  <si>
+    <t>incidencia_100k</t>
+  </si>
+  <si>
+    <t>mortalidade_100k</t>
+  </si>
+  <si>
+    <t>letalidade_pct</t>
+  </si>
+  <si>
+    <t>pct_uti</t>
+  </si>
+  <si>
+    <t>Nova Esperanca</t>
+  </si>
+  <si>
+    <t>Uniflor</t>
+  </si>
+  <si>
+    <t>Atalaia</t>
+  </si>
+  <si>
+    <t>Itaguaje</t>
+  </si>
+  <si>
+    <t>Ourizona</t>
+  </si>
+  <si>
+    <t>Nossa Senhora Das Gracas</t>
+  </si>
+  <si>
+    <t>Sao Jorge Do Ivai</t>
+  </si>
+  <si>
+    <t>Maringa</t>
+  </si>
+  <si>
+    <t>Santo Inacio</t>
+  </si>
+  <si>
+    <t>Colorado</t>
+  </si>
+  <si>
+    <t>Itambe</t>
+  </si>
+  <si>
+    <t>Florai</t>
+  </si>
+  <si>
+    <t>Marialva</t>
+  </si>
+  <si>
+    <t>Santa Ines</t>
+  </si>
+  <si>
+    <t>Paranacity</t>
+  </si>
+  <si>
+    <t>Sarandi</t>
+  </si>
+  <si>
+    <t>Astorga</t>
+  </si>
+  <si>
+    <t>Floresta</t>
+  </si>
+  <si>
+    <t>Munhoz De Melo</t>
+  </si>
+  <si>
+    <t>Mandaguacu</t>
+  </si>
+  <si>
+    <t>Paicandu</t>
+  </si>
+  <si>
+    <t>Presidente Castelo Branco</t>
+  </si>
+  <si>
+    <t>Santa Fe</t>
+  </si>
+  <si>
+    <t>Lobato</t>
+  </si>
+  <si>
+    <t>Florida</t>
+  </si>
+  <si>
+    <t>Iguaracu</t>
+  </si>
+  <si>
+    <t>Mandaguari</t>
+  </si>
+  <si>
+    <t>Doutor Camargo</t>
+  </si>
+  <si>
+    <t>variavel</t>
+  </si>
+  <si>
+    <t>pct_preenchido</t>
+  </si>
+  <si>
+    <t>n_total</t>
+  </si>
+  <si>
+    <t>Obesidade</t>
+  </si>
+  <si>
+    <t>Diabetes</t>
+  </si>
+  <si>
+    <t>Cardiopatia</t>
+  </si>
+  <si>
+    <t>Imunodepressão</t>
+  </si>
+  <si>
+    <t>Evolução (Desfecho)</t>
+  </si>
+  <si>
+    <t>Critério Confirmação</t>
+  </si>
+  <si>
+    <t>Bairro</t>
+  </si>
+  <si>
+    <t>Antiviral</t>
+  </si>
+  <si>
+    <t>Raça/Cor</t>
+  </si>
+  <si>
+    <t>Data Internação</t>
+  </si>
+  <si>
+    <t>Vacinação COVID</t>
+  </si>
+  <si>
+    <t>Sexo</t>
+  </si>
+  <si>
+    <t>Idade</t>
+  </si>
+  <si>
+    <t>Semana Epidemiológica</t>
+  </si>
+  <si>
+    <t>Data Início Sintomas</t>
+  </si>
+  <si>
+    <t>comorbidade</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>pct</t>
+  </si>
+  <si>
+    <t>Asma</t>
+  </si>
+  <si>
+    <t>Doença Neurológica</t>
+  </si>
+  <si>
+    <t>Pneumopatia</t>
+  </si>
+  <si>
+    <t>Doença Renal</t>
+  </si>
+  <si>
+    <t>Doença Hepática</t>
+  </si>
+  <si>
+    <t>Síndrome de Down</t>
+  </si>
+  <si>
+    <t>faixa_etaria</t>
+  </si>
+  <si>
+    <t>obitos</t>
+  </si>
+  <si>
+    <t>0-6 meses</t>
+  </si>
+  <si>
+    <t>1-4 anos</t>
+  </si>
+  <si>
+    <t>10-14 anos</t>
+  </si>
+  <si>
+    <t>15-19 anos</t>
+  </si>
+  <si>
+    <t>20-29 anos</t>
+  </si>
+  <si>
+    <t>30-39 anos</t>
+  </si>
+  <si>
+    <t>40-49 anos</t>
+  </si>
+  <si>
+    <t>5-9 anos</t>
+  </si>
+  <si>
+    <t>50-59 anos</t>
+  </si>
+  <si>
+    <t>6-11 meses</t>
+  </si>
+  <si>
+    <t>60 anos e mais</t>
+  </si>
+  <si>
+    <t>criterio_label</t>
+  </si>
+  <si>
+    <t>total</t>
+  </si>
+  <si>
+    <t>Laboratorial</t>
+  </si>
+  <si>
+    <t>Não informado</t>
+  </si>
+  <si>
+    <t>Clínico-Imagem</t>
+  </si>
+  <si>
+    <t>antiviral_label</t>
+  </si>
+  <si>
+    <t>Ignorado/Não registrado</t>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
+    <t>Sim</t>
+  </si>
+  <si>
+    <t>vacina_label</t>
+  </si>
+  <si>
+    <t>Não vacinado</t>
+  </si>
+  <si>
+    <t>Vacinado</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -361,53 +630,35 @@
   <dimension ref="A1:H29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>municipio</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>casos</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>obitos_srag</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>uti</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>incidencia_100k</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>mortalidade_100k</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>letalidade_pct</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>pct_uti</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Nova Esperanca</t>
-        </is>
+    <row r="1" spans="1:8" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>8</v>
       </c>
       <c r="B2">
         <v>98</v>
@@ -431,11 +682,9 @@
         <v>5.1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Uniflor</t>
-        </is>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>9</v>
       </c>
       <c r="B3">
         <v>6</v>
@@ -459,11 +708,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Atalaia</t>
-        </is>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>10</v>
       </c>
       <c r="B4">
         <v>9</v>
@@ -487,11 +734,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Itaguaje</t>
-        </is>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>11</v>
       </c>
       <c r="B5">
         <v>10</v>
@@ -515,11 +760,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ourizona</t>
-        </is>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>12</v>
       </c>
       <c r="B6">
         <v>7</v>
@@ -543,11 +786,9 @@
         <v>42.9</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Nossa Senhora Das Gracas</t>
-        </is>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>13</v>
       </c>
       <c r="B7">
         <v>8</v>
@@ -571,11 +812,9 @@
         <v>37.5</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Sao Jorge Do Ivai</t>
-        </is>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>14</v>
       </c>
       <c r="B8">
         <v>11</v>
@@ -599,39 +838,35 @@
         <v>27.3</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Maringa</t>
-        </is>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>15</v>
       </c>
       <c r="B9">
-        <v>829</v>
+        <v>836</v>
       </c>
       <c r="C9">
         <v>81</v>
       </c>
       <c r="D9">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E9">
-        <v>192.9</v>
+        <v>194.6</v>
       </c>
       <c r="F9">
         <v>18.9</v>
       </c>
       <c r="G9">
-        <v>9.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H9">
-        <v>28.3</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Santo Inacio</t>
-        </is>
+        <v>28.6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>16</v>
       </c>
       <c r="B10">
         <v>12</v>
@@ -655,11 +890,9 @@
         <v>16.7</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Colorado</t>
-        </is>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>17</v>
       </c>
       <c r="B11">
         <v>41</v>
@@ -683,11 +916,9 @@
         <v>4.9</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Itambe</t>
-        </is>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>18</v>
       </c>
       <c r="B12">
         <v>10</v>
@@ -711,11 +942,9 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Florai</t>
-        </is>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>19</v>
       </c>
       <c r="B13">
         <v>6</v>
@@ -739,14 +968,12 @@
         <v>16.7</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Marialva</t>
-        </is>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>20</v>
       </c>
       <c r="B14">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C14">
         <v>2</v>
@@ -755,23 +982,21 @@
         <v>25</v>
       </c>
       <c r="E14">
-        <v>120.7</v>
+        <v>122.9</v>
       </c>
       <c r="F14">
         <v>4.5</v>
       </c>
       <c r="G14">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="H14">
-        <v>46.3</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Santa Ines</t>
-        </is>
+        <v>45.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
+        <v>21</v>
       </c>
       <c r="B15">
         <v>2</v>
@@ -795,11 +1020,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Paranacity</t>
-        </is>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>22</v>
       </c>
       <c r="B16">
         <v>10</v>
@@ -823,39 +1046,35 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Sarandi</t>
-        </is>
+    <row r="17" spans="1:8">
+      <c r="A17" t="s">
+        <v>23</v>
       </c>
       <c r="B17">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C17">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D17">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E17">
-        <v>84.3</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="F17">
-        <v>5.5</v>
+        <v>6.2</v>
       </c>
       <c r="G17">
-        <v>6.5</v>
+        <v>7.1</v>
       </c>
       <c r="H17">
-        <v>38.9</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Astorga</t>
-        </is>
+        <v>38.4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" t="s">
+        <v>24</v>
       </c>
       <c r="B18">
         <v>14</v>
@@ -879,11 +1098,9 @@
         <v>35.7</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Floresta</t>
-        </is>
+    <row r="19" spans="1:8">
+      <c r="A19" t="s">
+        <v>25</v>
       </c>
       <c r="B19">
         <v>6</v>
@@ -907,11 +1124,9 @@
         <v>16.7</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Munhoz De Melo</t>
-        </is>
+    <row r="20" spans="1:8">
+      <c r="A20" t="s">
+        <v>26</v>
       </c>
       <c r="B20">
         <v>2</v>
@@ -935,11 +1150,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Mandaguacu</t>
-        </is>
+    <row r="21" spans="1:8">
+      <c r="A21" t="s">
+        <v>27</v>
       </c>
       <c r="B21">
         <v>17</v>
@@ -963,67 +1176,61 @@
         <v>41.2</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Presidente Castelo Branco</t>
-        </is>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
+        <v>28</v>
       </c>
       <c r="B22">
+        <v>23</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22">
+        <v>14</v>
+      </c>
+      <c r="E22">
+        <v>47.2</v>
+      </c>
+      <c r="F22">
+        <v>2.1</v>
+      </c>
+      <c r="G22">
+        <v>4.3</v>
+      </c>
+      <c r="H22">
+        <v>60.9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23">
         <v>2</v>
       </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22">
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
         <v>46.5</v>
       </c>
-      <c r="F22">
-        <v>0</v>
-      </c>
-      <c r="G22">
-        <v>0</v>
-      </c>
-      <c r="H22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Paicandu</t>
-        </is>
-      </c>
-      <c r="B23">
-        <v>22</v>
-      </c>
-      <c r="C23">
-        <v>1</v>
-      </c>
-      <c r="D23">
-        <v>13</v>
-      </c>
-      <c r="E23">
-        <v>45.2</v>
-      </c>
       <c r="F23">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="H23">
-        <v>59.1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Santa Fe</t>
-        </is>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" t="s">
+        <v>30</v>
       </c>
       <c r="B24">
         <v>5</v>
@@ -1047,11 +1254,9 @@
         <v>80</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Lobato</t>
-        </is>
+    <row r="25" spans="1:8">
+      <c r="A25" t="s">
+        <v>31</v>
       </c>
       <c r="B25">
         <v>2</v>
@@ -1075,11 +1280,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Florida</t>
-        </is>
+    <row r="26" spans="1:8">
+      <c r="A26" t="s">
+        <v>32</v>
       </c>
       <c r="B26">
         <v>1</v>
@@ -1103,11 +1306,9 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Iguaracu</t>
-        </is>
+    <row r="27" spans="1:8">
+      <c r="A27" t="s">
+        <v>33</v>
       </c>
       <c r="B27">
         <v>2</v>
@@ -1131,11 +1332,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Mandaguari</t>
-        </is>
+    <row r="28" spans="1:8">
+      <c r="A28" t="s">
+        <v>34</v>
       </c>
       <c r="B28">
         <v>13</v>
@@ -1159,11 +1358,9 @@
         <v>76.90000000000001</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Doutor Camargo</t>
-        </is>
+    <row r="29" spans="1:8">
+      <c r="A29" t="s">
+        <v>35</v>
       </c>
       <c r="B29">
         <v>2</v>
@@ -1197,216 +1394,180 @@
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>variavel</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>pct_preenchido</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>n_total</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Obesidade</t>
-        </is>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>39</v>
       </c>
       <c r="B2">
         <v>59.9</v>
       </c>
       <c r="C2">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Diabetes</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>40</v>
       </c>
       <c r="B3">
         <v>60.4</v>
       </c>
       <c r="C3">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Cardiopatia</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>41</v>
       </c>
       <c r="B4">
         <v>60.5</v>
       </c>
       <c r="C4">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Imunodepressão</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>42</v>
       </c>
       <c r="B5">
         <v>60.5</v>
       </c>
       <c r="C5">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Evolução (Desfecho)</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>43</v>
       </c>
       <c r="B6">
-        <v>79.5</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="C6">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Critério Confirmação</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>44</v>
       </c>
       <c r="B7">
-        <v>86.90000000000001</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="C7">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Bairro</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>45</v>
       </c>
       <c r="B8">
-        <v>89.90000000000001</v>
+        <v>90</v>
       </c>
       <c r="C8">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Antiviral</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>46</v>
       </c>
       <c r="B9">
-        <v>97.59999999999999</v>
+        <v>98</v>
       </c>
       <c r="C9">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Raça/Cor</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>47</v>
       </c>
       <c r="B10">
         <v>98.5</v>
       </c>
       <c r="C10">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Data Internação</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>48</v>
       </c>
       <c r="B11">
-        <v>99</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="C11">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Vacinação COVID</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>49</v>
       </c>
       <c r="B12">
         <v>99.8</v>
       </c>
       <c r="C12">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Sexo</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>50</v>
       </c>
       <c r="B13">
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Idade</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>51</v>
       </c>
       <c r="B14">
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Semana Epidemiológica</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>52</v>
       </c>
       <c r="B15">
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1309</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Data Início Sintomas</t>
-        </is>
+        <v>1322</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>53</v>
       </c>
       <c r="B16">
         <v>100</v>
       </c>
       <c r="C16">
-        <v>1309</v>
+        <v>1322</v>
       </c>
     </row>
   </sheetData>
@@ -1419,106 +1580,86 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>comorbidade</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Cardiopatia</t>
-        </is>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>41</v>
       </c>
       <c r="B2">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="C2">
-        <v>29.6</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Diabetes</t>
-        </is>
+        <v>29.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>40</v>
       </c>
       <c r="B3">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C3">
-        <v>14.9</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Asma</t>
-        </is>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>57</v>
       </c>
       <c r="B4">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C4">
         <v>12.6</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Doença Neurológica</t>
-        </is>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>58</v>
       </c>
       <c r="B5">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C5">
-        <v>11.5</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Pneumopatia</t>
-        </is>
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>59</v>
       </c>
       <c r="B6">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C6">
         <v>10.8</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Doença Renal</t>
-        </is>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>60</v>
       </c>
       <c r="B7">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C7">
-        <v>3.4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Obesidade</t>
-        </is>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>39</v>
       </c>
       <c r="B8">
         <v>34</v>
@@ -1527,24 +1668,20 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Imunodepressão</t>
-        </is>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>42</v>
       </c>
       <c r="B9">
         <v>27</v>
       </c>
       <c r="C9">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Doença Hepática</t>
-        </is>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>61</v>
       </c>
       <c r="B10">
         <v>10</v>
@@ -1553,11 +1690,9 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Síndrome de Down</t>
-        </is>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>62</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -1576,36 +1711,26 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>faixa_etaria</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>casos</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>obitos</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>letalidade_pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>0-6 meses</t>
-        </is>
+    <row r="1" spans="1:4" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>65</v>
       </c>
       <c r="B2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -1614,14 +1739,12 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1-4 anos</t>
-        </is>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>66</v>
       </c>
       <c r="B3">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1630,11 +1753,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>10-14 anos</t>
-        </is>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>67</v>
       </c>
       <c r="B4">
         <v>29</v>
@@ -1646,11 +1767,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>15-19 anos</t>
-        </is>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>68</v>
       </c>
       <c r="B5">
         <v>7</v>
@@ -1662,11 +1781,9 @@
         <v>28.6</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>20-29 anos</t>
-        </is>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>69</v>
       </c>
       <c r="B6">
         <v>21</v>
@@ -1678,27 +1795,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>30-39 anos</t>
-        </is>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>70</v>
       </c>
       <c r="B7">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
       <c r="D7">
-        <v>6.2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>40-49 anos</t>
-        </is>
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>71</v>
       </c>
       <c r="B8">
         <v>43</v>
@@ -1710,11 +1823,9 @@
         <v>2.3</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>5-9 anos</t>
-        </is>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>72</v>
       </c>
       <c r="B9">
         <v>77</v>
@@ -1726,30 +1837,26 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>50-59 anos</t>
-        </is>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>73</v>
       </c>
       <c r="B10">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C10">
         <v>8</v>
       </c>
       <c r="D10">
-        <v>11.6</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>6-11 meses</t>
-        </is>
+        <v>11.3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>74</v>
       </c>
       <c r="B11">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1758,17 +1865,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>60 anos e mais</t>
-        </is>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>75</v>
       </c>
       <c r="B12">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="C12">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D12">
         <v>14.6</v>
@@ -1784,65 +1889,51 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>faixa_etaria</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>casos</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>uti</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>pct_uti</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>0-6 meses</t>
-        </is>
+    <row r="1" spans="1:4" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>65</v>
       </c>
       <c r="B2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D2">
-        <v>44.4</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1-4 anos</t>
-        </is>
+        <v>44.9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>66</v>
       </c>
       <c r="B3">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C3">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>10-14 anos</t>
-        </is>
+        <v>20.4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>67</v>
       </c>
       <c r="B4">
         <v>29</v>
@@ -1854,11 +1945,9 @@
         <v>17.2</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>15-19 anos</t>
-        </is>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>68</v>
       </c>
       <c r="B5">
         <v>7</v>
@@ -1870,11 +1959,9 @@
         <v>28.6</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>20-29 anos</t>
-        </is>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>69</v>
       </c>
       <c r="B6">
         <v>21</v>
@@ -1886,27 +1973,23 @@
         <v>33.3</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>30-39 anos</t>
-        </is>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>70</v>
       </c>
       <c r="B7">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7">
         <v>10</v>
       </c>
       <c r="D7">
-        <v>31.2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>40-49 anos</t>
-        </is>
+        <v>30.3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>71</v>
       </c>
       <c r="B8">
         <v>43</v>
@@ -1918,11 +2001,9 @@
         <v>34.9</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>5-9 anos</t>
-        </is>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>72</v>
       </c>
       <c r="B9">
         <v>77</v>
@@ -1934,52 +2015,46 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>50-59 anos</t>
-        </is>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>73</v>
       </c>
       <c r="B10">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C10">
         <v>23</v>
       </c>
       <c r="D10">
-        <v>33.3</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>6-11 meses</t>
-        </is>
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>74</v>
       </c>
       <c r="B11">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C11">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D11">
-        <v>24.5</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>60 anos e mais</t>
-        </is>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>75</v>
       </c>
       <c r="B12">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="C12">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D12">
-        <v>28</v>
+        <v>28.2</v>
       </c>
     </row>
   </sheetData>
@@ -1992,54 +2067,42 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>criterio_label</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Laboratorial</t>
-        </is>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>78</v>
       </c>
       <c r="B2">
-        <v>718</v>
+        <v>738</v>
       </c>
       <c r="C2">
-        <v>98.8</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Não informado</t>
-        </is>
+        <v>98.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>79</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Clínico-Imagem</t>
-        </is>
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>80</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -2058,60 +2121,48 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>antiviral_label</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Ignorado/Não registrado</t>
-        </is>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>82</v>
       </c>
       <c r="B2">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C2">
-        <v>2.4</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>83</v>
       </c>
       <c r="B3">
-        <v>950</v>
+        <v>963</v>
       </c>
       <c r="C3">
-        <v>72.59999999999999</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
+        <v>72.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>84</v>
       </c>
       <c r="B4">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="C4">
-        <v>25</v>
+        <v>25.1</v>
       </c>
     </row>
   </sheetData>
@@ -2124,28 +2175,20 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>vacina_label</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>total</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Ignorado/Não registrado</t>
-        </is>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>82</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -2154,30 +2197,26 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Não vacinado</t>
-        </is>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>86</v>
       </c>
       <c r="B3">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="C3">
-        <v>40.4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Vacinado</t>
-        </is>
+        <v>40.3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>87</v>
       </c>
       <c r="B4">
-        <v>778</v>
+        <v>787</v>
       </c>
       <c r="C4">
-        <v>59.4</v>
+        <v>59.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização de dados — 25/08/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -53,15 +53,18 @@
     <t>Uniflor</t>
   </si>
   <si>
+    <t>Ourizona</t>
+  </si>
+  <si>
+    <t>Santa Ines</t>
+  </si>
+  <si>
     <t>Atalaia</t>
   </si>
   <si>
     <t>Itaguaje</t>
   </si>
   <si>
-    <t>Ourizona</t>
-  </si>
-  <si>
     <t>Nossa Senhora Das Gracas</t>
   </si>
   <si>
@@ -80,15 +83,12 @@
     <t>Itambe</t>
   </si>
   <si>
+    <t>Marialva</t>
+  </si>
+  <si>
     <t>Florai</t>
   </si>
   <si>
-    <t>Marialva</t>
-  </si>
-  <si>
-    <t>Santa Ines</t>
-  </si>
-  <si>
     <t>Paranacity</t>
   </si>
   <si>
@@ -155,10 +155,10 @@
     <t>Evolução (Desfecho)</t>
   </si>
   <si>
+    <t>Bairro</t>
+  </si>
+  <si>
     <t>Critério Confirmação</t>
-  </si>
-  <si>
-    <t>Bairro</t>
   </si>
   <si>
     <t>Antiviral</t>
@@ -661,7 +661,7 @@
         <v>8</v>
       </c>
       <c r="B2">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C2">
         <v>5</v>
@@ -670,7 +670,7 @@
         <v>5</v>
       </c>
       <c r="E2">
-        <v>361.1</v>
+        <v>364.7</v>
       </c>
       <c r="F2">
         <v>18.4</v>
@@ -713,16 +713,16 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E4">
-        <v>222.4</v>
+        <v>250.5</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -731,7 +731,7 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -739,25 +739,25 @@
         <v>11</v>
       </c>
       <c r="B5">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>220.8</v>
+        <v>229.2</v>
       </c>
       <c r="F5">
-        <v>22.1</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -765,16 +765,16 @@
         <v>12</v>
       </c>
       <c r="B6">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>219.2</v>
+        <v>222.4</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -783,7 +783,7 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>42.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -791,25 +791,25 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7">
-        <v>218</v>
+        <v>220.8</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>22.1</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H7">
-        <v>37.5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -817,25 +817,25 @@
         <v>14</v>
       </c>
       <c r="B8">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8">
         <v>3</v>
       </c>
       <c r="E8">
-        <v>212.8</v>
+        <v>218</v>
       </c>
       <c r="F8">
-        <v>19.3</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>9.1</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>27.3</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -843,25 +843,25 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>836</v>
+        <v>11</v>
       </c>
       <c r="C9">
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="D9">
-        <v>239</v>
+        <v>3</v>
       </c>
       <c r="E9">
-        <v>194.6</v>
+        <v>212.8</v>
       </c>
       <c r="F9">
-        <v>18.9</v>
+        <v>19.3</v>
       </c>
       <c r="G9">
-        <v>9.699999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="H9">
-        <v>28.6</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -869,25 +869,25 @@
         <v>16</v>
       </c>
       <c r="B10">
-        <v>12</v>
+        <v>855</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="D10">
-        <v>2</v>
+        <v>243</v>
       </c>
       <c r="E10">
-        <v>185.7</v>
+        <v>199</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>19.8</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>9.9</v>
       </c>
       <c r="H10">
-        <v>16.7</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -895,7 +895,7 @@
         <v>17</v>
       </c>
       <c r="B11">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -904,7 +904,7 @@
         <v>2</v>
       </c>
       <c r="E11">
-        <v>175.9</v>
+        <v>185.7</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -913,7 +913,7 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>4.9</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -921,7 +921,7 @@
         <v>18</v>
       </c>
       <c r="B12">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -930,7 +930,7 @@
         <v>2</v>
       </c>
       <c r="E12">
-        <v>160.6</v>
+        <v>175.9</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -939,7 +939,7 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>20</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -947,16 +947,16 @@
         <v>19</v>
       </c>
       <c r="B13">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C13">
         <v>0</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13">
-        <v>124.9</v>
+        <v>160.6</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -965,7 +965,7 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>16.7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -973,25 +973,25 @@
         <v>20</v>
       </c>
       <c r="B14">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C14">
         <v>2</v>
       </c>
       <c r="D14">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E14">
-        <v>122.9</v>
+        <v>127.4</v>
       </c>
       <c r="F14">
         <v>4.5</v>
       </c>
       <c r="G14">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="H14">
-        <v>45.5</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -999,16 +999,16 @@
         <v>21</v>
       </c>
       <c r="B15">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C15">
         <v>0</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15">
-        <v>114.6</v>
+        <v>124.9</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -1017,7 +1017,7 @@
         <v>0</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1051,16 +1051,16 @@
         <v>23</v>
       </c>
       <c r="B17">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C17">
         <v>8</v>
       </c>
       <c r="D17">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E17">
-        <v>87.40000000000001</v>
+        <v>88.2</v>
       </c>
       <c r="F17">
         <v>6.2</v>
@@ -1069,7 +1069,7 @@
         <v>7.1</v>
       </c>
       <c r="H17">
-        <v>38.4</v>
+        <v>38.9</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1413,7 +1413,7 @@
         <v>59.9</v>
       </c>
       <c r="C2">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1421,10 +1421,10 @@
         <v>40</v>
       </c>
       <c r="B3">
-        <v>60.4</v>
+        <v>60.3</v>
       </c>
       <c r="C3">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1435,7 +1435,7 @@
         <v>60.5</v>
       </c>
       <c r="C4">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1446,7 +1446,7 @@
         <v>60.5</v>
       </c>
       <c r="C5">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1454,10 +1454,10 @@
         <v>43</v>
       </c>
       <c r="B6">
-        <v>82.40000000000001</v>
+        <v>83.2</v>
       </c>
       <c r="C6">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1465,10 +1465,10 @@
         <v>44</v>
       </c>
       <c r="B7">
-        <v>89.40000000000001</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="C7">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1476,10 +1476,10 @@
         <v>45</v>
       </c>
       <c r="B8">
-        <v>90</v>
+        <v>90.3</v>
       </c>
       <c r="C8">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1487,10 +1487,10 @@
         <v>46</v>
       </c>
       <c r="B9">
-        <v>98</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="C9">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1501,7 +1501,7 @@
         <v>98.5</v>
       </c>
       <c r="C10">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1512,7 +1512,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="C11">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1520,10 +1520,10 @@
         <v>49</v>
       </c>
       <c r="B12">
-        <v>99.8</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="C12">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1534,7 +1534,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1545,7 +1545,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1556,7 +1556,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1567,7 +1567,7 @@
         <v>100</v>
       </c>
       <c r="C16">
-        <v>1322</v>
+        <v>1348</v>
       </c>
     </row>
   </sheetData>
@@ -1596,7 +1596,7 @@
         <v>41</v>
       </c>
       <c r="B2">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="C2">
         <v>29.7</v>
@@ -1607,10 +1607,10 @@
         <v>40</v>
       </c>
       <c r="B3">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C3">
-        <v>15</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1618,10 +1618,10 @@
         <v>57</v>
       </c>
       <c r="B4">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C4">
-        <v>12.6</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1629,10 +1629,10 @@
         <v>58</v>
       </c>
       <c r="B5">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C5">
-        <v>11.6</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1640,7 +1640,7 @@
         <v>59</v>
       </c>
       <c r="B6">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C6">
         <v>10.8</v>
@@ -1651,7 +1651,7 @@
         <v>60</v>
       </c>
       <c r="B7">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C7">
         <v>3.5</v>
@@ -1665,7 +1665,7 @@
         <v>34</v>
       </c>
       <c r="C8">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1684,7 +1684,7 @@
         <v>61</v>
       </c>
       <c r="B10">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C10">
         <v>0.8</v>
@@ -1698,7 +1698,7 @@
         <v>10</v>
       </c>
       <c r="C11">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
   </sheetData>
@@ -1730,7 +1730,7 @@
         <v>65</v>
       </c>
       <c r="B2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -1744,7 +1744,7 @@
         <v>66</v>
       </c>
       <c r="B3">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1758,7 +1758,7 @@
         <v>67</v>
       </c>
       <c r="B4">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1800,13 +1800,13 @@
         <v>70</v>
       </c>
       <c r="B7">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
       <c r="D7">
-        <v>6.1</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1814,7 +1814,7 @@
         <v>71</v>
       </c>
       <c r="B8">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1842,13 +1842,13 @@
         <v>73</v>
       </c>
       <c r="B10">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C10">
         <v>8</v>
       </c>
       <c r="D10">
-        <v>11.3</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -1856,7 +1856,7 @@
         <v>74</v>
       </c>
       <c r="B11">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1870,13 +1870,13 @@
         <v>75</v>
       </c>
       <c r="B12">
-        <v>581</v>
+        <v>596</v>
       </c>
       <c r="C12">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D12">
-        <v>14.6</v>
+        <v>14.9</v>
       </c>
     </row>
   </sheetData>
@@ -1908,13 +1908,13 @@
         <v>65</v>
       </c>
       <c r="B2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C2">
         <v>57</v>
       </c>
       <c r="D2">
-        <v>44.9</v>
+        <v>44.5</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1922,13 +1922,13 @@
         <v>66</v>
       </c>
       <c r="B3">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C3">
         <v>45</v>
       </c>
       <c r="D3">
-        <v>20.4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1936,13 +1936,13 @@
         <v>67</v>
       </c>
       <c r="B4">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4">
         <v>5</v>
       </c>
       <c r="D4">
-        <v>17.2</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1978,13 +1978,13 @@
         <v>70</v>
       </c>
       <c r="B7">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D7">
-        <v>30.3</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1992,13 +1992,13 @@
         <v>71</v>
       </c>
       <c r="B8">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C8">
         <v>15</v>
       </c>
       <c r="D8">
-        <v>34.9</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2020,13 +2020,13 @@
         <v>73</v>
       </c>
       <c r="B10">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C10">
         <v>23</v>
       </c>
       <c r="D10">
-        <v>32.4</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2034,13 +2034,13 @@
         <v>74</v>
       </c>
       <c r="B11">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C11">
         <v>28</v>
       </c>
       <c r="D11">
-        <v>25</v>
+        <v>24.6</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2048,13 +2048,13 @@
         <v>75</v>
       </c>
       <c r="B12">
-        <v>581</v>
+        <v>596</v>
       </c>
       <c r="C12">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="D12">
-        <v>28.2</v>
+        <v>28.5</v>
       </c>
     </row>
   </sheetData>
@@ -2083,7 +2083,7 @@
         <v>78</v>
       </c>
       <c r="B2">
-        <v>738</v>
+        <v>754</v>
       </c>
       <c r="C2">
         <v>98.7</v>
@@ -2097,7 +2097,7 @@
         <v>8</v>
       </c>
       <c r="C3">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2137,10 +2137,10 @@
         <v>82</v>
       </c>
       <c r="B2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2148,10 +2148,10 @@
         <v>83</v>
       </c>
       <c r="B3">
-        <v>963</v>
+        <v>974</v>
       </c>
       <c r="C3">
-        <v>72.8</v>
+        <v>72.3</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2159,10 +2159,10 @@
         <v>84</v>
       </c>
       <c r="B4">
-        <v>332</v>
+        <v>346</v>
       </c>
       <c r="C4">
-        <v>25.1</v>
+        <v>25.7</v>
       </c>
     </row>
   </sheetData>
@@ -2194,7 +2194,7 @@
         <v>2</v>
       </c>
       <c r="C2">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2202,10 +2202,10 @@
         <v>86</v>
       </c>
       <c r="B3">
-        <v>533</v>
+        <v>541</v>
       </c>
       <c r="C3">
-        <v>40.3</v>
+        <v>40.1</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2213,10 +2213,10 @@
         <v>87</v>
       </c>
       <c r="B4">
-        <v>787</v>
+        <v>805</v>
       </c>
       <c r="C4">
-        <v>59.5</v>
+        <v>59.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização de dados — 27/08/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -83,12 +83,12 @@
     <t>Itambe</t>
   </si>
   <si>
+    <t>Florai</t>
+  </si>
+  <si>
     <t>Marialva</t>
   </si>
   <si>
-    <t>Florai</t>
-  </si>
-  <si>
     <t>Paranacity</t>
   </si>
   <si>
@@ -122,10 +122,10 @@
     <t>Florida</t>
   </si>
   <si>
+    <t>Mandaguari</t>
+  </si>
+  <si>
     <t>Iguaracu</t>
-  </si>
-  <si>
-    <t>Mandaguari</t>
   </si>
   <si>
     <t>Doutor Camargo</t>
@@ -664,7 +664,7 @@
         <v>99</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D2">
         <v>5</v>
@@ -673,10 +673,10 @@
         <v>364.7</v>
       </c>
       <c r="F2">
-        <v>18.4</v>
+        <v>36.8</v>
       </c>
       <c r="G2">
-        <v>5.1</v>
+        <v>10.1</v>
       </c>
       <c r="H2">
         <v>5.1</v>
@@ -869,25 +869,25 @@
         <v>16</v>
       </c>
       <c r="B10">
-        <v>855</v>
+        <v>863</v>
       </c>
       <c r="C10">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D10">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E10">
-        <v>199</v>
+        <v>200.9</v>
       </c>
       <c r="F10">
-        <v>19.8</v>
+        <v>20.2</v>
       </c>
       <c r="G10">
-        <v>9.9</v>
+        <v>10.1</v>
       </c>
       <c r="H10">
-        <v>28.4</v>
+        <v>28.3</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -921,7 +921,7 @@
         <v>18</v>
       </c>
       <c r="B12">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -930,7 +930,7 @@
         <v>2</v>
       </c>
       <c r="E12">
-        <v>175.9</v>
+        <v>180.2</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -939,7 +939,7 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -973,25 +973,25 @@
         <v>20</v>
       </c>
       <c r="B14">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
         <v>2</v>
       </c>
-      <c r="D14">
-        <v>27</v>
-      </c>
       <c r="E14">
-        <v>127.4</v>
+        <v>145.7</v>
       </c>
       <c r="F14">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="H14">
-        <v>47.4</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -999,25 +999,25 @@
         <v>21</v>
       </c>
       <c r="B15">
-        <v>6</v>
+        <v>58</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="E15">
-        <v>124.9</v>
+        <v>129.6</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="H15">
-        <v>16.7</v>
+        <v>46.6</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1051,25 +1051,25 @@
         <v>23</v>
       </c>
       <c r="B17">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C17">
         <v>8</v>
       </c>
       <c r="D17">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E17">
-        <v>88.2</v>
+        <v>89</v>
       </c>
       <c r="F17">
         <v>6.2</v>
       </c>
       <c r="G17">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="H17">
-        <v>38.9</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1210,7 +1210,7 @@
         <v>2</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -1219,10 +1219,10 @@
         <v>46.5</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>23.2</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H23">
         <v>0</v>
@@ -1311,16 +1311,16 @@
         <v>33</v>
       </c>
       <c r="B27">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C27">
         <v>0</v>
       </c>
       <c r="D27">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E27">
-        <v>35.1</v>
+        <v>36.5</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -1329,7 +1329,7 @@
         <v>0</v>
       </c>
       <c r="H27">
-        <v>50</v>
+        <v>78.59999999999999</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1337,16 +1337,16 @@
         <v>34</v>
       </c>
       <c r="B28">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C28">
         <v>0</v>
       </c>
       <c r="D28">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E28">
-        <v>33.9</v>
+        <v>35.1</v>
       </c>
       <c r="F28">
         <v>0</v>
@@ -1355,7 +1355,7 @@
         <v>0</v>
       </c>
       <c r="H28">
-        <v>76.90000000000001</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1410,10 +1410,10 @@
         <v>39</v>
       </c>
       <c r="B2">
-        <v>59.9</v>
+        <v>60.2</v>
       </c>
       <c r="C2">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1421,10 +1421,10 @@
         <v>40</v>
       </c>
       <c r="B3">
-        <v>60.3</v>
+        <v>60.6</v>
       </c>
       <c r="C3">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1432,10 +1432,10 @@
         <v>41</v>
       </c>
       <c r="B4">
-        <v>60.5</v>
+        <v>60.8</v>
       </c>
       <c r="C4">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1443,10 +1443,10 @@
         <v>42</v>
       </c>
       <c r="B5">
-        <v>60.5</v>
+        <v>60.8</v>
       </c>
       <c r="C5">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1454,10 +1454,10 @@
         <v>43</v>
       </c>
       <c r="B6">
-        <v>83.2</v>
+        <v>87.2</v>
       </c>
       <c r="C6">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1468,7 +1468,7 @@
         <v>90.09999999999999</v>
       </c>
       <c r="C7">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1476,10 +1476,10 @@
         <v>45</v>
       </c>
       <c r="B8">
-        <v>90.3</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="C8">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1487,10 +1487,10 @@
         <v>46</v>
       </c>
       <c r="B9">
-        <v>97.90000000000001</v>
+        <v>98</v>
       </c>
       <c r="C9">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1501,7 +1501,7 @@
         <v>98.5</v>
       </c>
       <c r="C10">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1512,7 +1512,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="C11">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1523,7 +1523,7 @@
         <v>99.90000000000001</v>
       </c>
       <c r="C12">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1534,7 +1534,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1545,7 +1545,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1556,7 +1556,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1567,7 +1567,7 @@
         <v>100</v>
       </c>
       <c r="C16">
-        <v>1348</v>
+        <v>1361</v>
       </c>
     </row>
   </sheetData>
@@ -1596,10 +1596,10 @@
         <v>41</v>
       </c>
       <c r="B2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C2">
-        <v>29.7</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1607,7 +1607,7 @@
         <v>40</v>
       </c>
       <c r="B3">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C3">
         <v>15.1</v>
@@ -1618,10 +1618,10 @@
         <v>57</v>
       </c>
       <c r="B4">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C4">
-        <v>12.4</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1629,10 +1629,10 @@
         <v>58</v>
       </c>
       <c r="B5">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C5">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1640,10 +1640,10 @@
         <v>59</v>
       </c>
       <c r="B6">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C6">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1733,10 +1733,10 @@
         <v>128</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1744,7 +1744,7 @@
         <v>66</v>
       </c>
       <c r="B3">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1758,7 +1758,7 @@
         <v>67</v>
       </c>
       <c r="B4">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1800,13 +1800,13 @@
         <v>70</v>
       </c>
       <c r="B7">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
       <c r="D7">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1828,7 +1828,7 @@
         <v>72</v>
       </c>
       <c r="B9">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1842,13 +1842,13 @@
         <v>73</v>
       </c>
       <c r="B10">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D10">
-        <v>11.1</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -1856,7 +1856,7 @@
         <v>74</v>
       </c>
       <c r="B11">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1870,13 +1870,13 @@
         <v>75</v>
       </c>
       <c r="B12">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="C12">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="D12">
-        <v>14.9</v>
+        <v>15.8</v>
       </c>
     </row>
   </sheetData>
@@ -1922,13 +1922,13 @@
         <v>66</v>
       </c>
       <c r="B3">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C3">
         <v>45</v>
       </c>
       <c r="D3">
-        <v>20</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1936,13 +1936,13 @@
         <v>67</v>
       </c>
       <c r="B4">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C4">
         <v>5</v>
       </c>
       <c r="D4">
-        <v>16.7</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1978,13 +1978,13 @@
         <v>70</v>
       </c>
       <c r="B7">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C7">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7">
-        <v>32.4</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2006,13 +2006,13 @@
         <v>72</v>
       </c>
       <c r="B9">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C9">
         <v>20</v>
       </c>
       <c r="D9">
-        <v>26</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2020,13 +2020,13 @@
         <v>73</v>
       </c>
       <c r="B10">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C10">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D10">
-        <v>31.9</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2034,13 +2034,13 @@
         <v>74</v>
       </c>
       <c r="B11">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C11">
         <v>28</v>
       </c>
       <c r="D11">
-        <v>24.6</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2048,13 +2048,13 @@
         <v>75</v>
       </c>
       <c r="B12">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="C12">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D12">
-        <v>28.5</v>
+        <v>28.4</v>
       </c>
     </row>
   </sheetData>
@@ -2083,10 +2083,10 @@
         <v>78</v>
       </c>
       <c r="B2">
-        <v>754</v>
+        <v>788</v>
       </c>
       <c r="C2">
-        <v>98.7</v>
+        <v>98.59999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2094,10 +2094,10 @@
         <v>79</v>
       </c>
       <c r="B3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2137,10 +2137,10 @@
         <v>82</v>
       </c>
       <c r="B2">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2148,7 +2148,7 @@
         <v>83</v>
       </c>
       <c r="B3">
-        <v>974</v>
+        <v>984</v>
       </c>
       <c r="C3">
         <v>72.3</v>
@@ -2159,7 +2159,7 @@
         <v>84</v>
       </c>
       <c r="B4">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C4">
         <v>25.7</v>
@@ -2202,10 +2202,10 @@
         <v>86</v>
       </c>
       <c r="B3">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="C3">
-        <v>40.1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2213,10 +2213,10 @@
         <v>87</v>
       </c>
       <c r="B4">
-        <v>805</v>
+        <v>815</v>
       </c>
       <c r="C4">
-        <v>59.7</v>
+        <v>59.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização de dados — 13/09/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -122,12 +122,12 @@
     <t>Florida</t>
   </si>
   <si>
+    <t>Iguaracu</t>
+  </si>
+  <si>
     <t>Mandaguari</t>
   </si>
   <si>
-    <t>Iguaracu</t>
-  </si>
-  <si>
     <t>Doutor Camargo</t>
   </si>
   <si>
@@ -140,6 +140,9 @@
     <t>n_total</t>
   </si>
   <si>
+    <t>Bairro</t>
+  </si>
+  <si>
     <t>Obesidade</t>
   </si>
   <si>
@@ -153,9 +156,6 @@
   </si>
   <si>
     <t>Evolução (Desfecho)</t>
-  </si>
-  <si>
-    <t>Bairro</t>
   </si>
   <si>
     <t>Critério Confirmação</t>
@@ -661,25 +661,25 @@
         <v>8</v>
       </c>
       <c r="B2">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C2">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2">
-        <v>364.7</v>
+        <v>361.1</v>
       </c>
       <c r="F2">
-        <v>36.8</v>
+        <v>14.7</v>
       </c>
       <c r="G2">
-        <v>10.1</v>
+        <v>4.1</v>
       </c>
       <c r="H2">
-        <v>5.1</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -869,22 +869,22 @@
         <v>16</v>
       </c>
       <c r="B10">
-        <v>863</v>
+        <v>837</v>
       </c>
       <c r="C10">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D10">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="E10">
-        <v>200.9</v>
+        <v>194.8</v>
       </c>
       <c r="F10">
-        <v>20.2</v>
+        <v>19.1</v>
       </c>
       <c r="G10">
-        <v>10.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H10">
         <v>28.3</v>
@@ -921,7 +921,7 @@
         <v>18</v>
       </c>
       <c r="B12">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -930,7 +930,7 @@
         <v>2</v>
       </c>
       <c r="E12">
-        <v>180.2</v>
+        <v>175.9</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -939,7 +939,7 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -947,7 +947,7 @@
         <v>19</v>
       </c>
       <c r="B13">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -956,7 +956,7 @@
         <v>2</v>
       </c>
       <c r="E13">
-        <v>160.6</v>
+        <v>144.5</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -965,7 +965,7 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>20</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -973,16 +973,16 @@
         <v>20</v>
       </c>
       <c r="B14">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C14">
         <v>0</v>
       </c>
       <c r="D14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14">
-        <v>145.7</v>
+        <v>124.9</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -991,7 +991,7 @@
         <v>0</v>
       </c>
       <c r="H14">
-        <v>28.6</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -999,25 +999,25 @@
         <v>21</v>
       </c>
       <c r="B15">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C15">
         <v>2</v>
       </c>
       <c r="D15">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E15">
-        <v>129.6</v>
+        <v>122.9</v>
       </c>
       <c r="F15">
         <v>4.5</v>
       </c>
       <c r="G15">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="H15">
-        <v>46.6</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1051,25 +1051,25 @@
         <v>23</v>
       </c>
       <c r="B17">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C17">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D17">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E17">
-        <v>89</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="F17">
+        <v>5.5</v>
+      </c>
+      <c r="G17">
         <v>6.2</v>
       </c>
-      <c r="G17">
-        <v>7</v>
-      </c>
       <c r="H17">
-        <v>39.5</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1210,7 +1210,7 @@
         <v>2</v>
       </c>
       <c r="C23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -1219,10 +1219,10 @@
         <v>46.5</v>
       </c>
       <c r="F23">
-        <v>23.2</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="H23">
         <v>0</v>
@@ -1311,16 +1311,16 @@
         <v>33</v>
       </c>
       <c r="B27">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="C27">
         <v>0</v>
       </c>
       <c r="D27">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E27">
-        <v>36.5</v>
+        <v>35.1</v>
       </c>
       <c r="F27">
         <v>0</v>
@@ -1329,7 +1329,7 @@
         <v>0</v>
       </c>
       <c r="H27">
-        <v>78.59999999999999</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1337,16 +1337,16 @@
         <v>34</v>
       </c>
       <c r="B28">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C28">
         <v>0</v>
       </c>
       <c r="D28">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E28">
-        <v>35.1</v>
+        <v>33.9</v>
       </c>
       <c r="F28">
         <v>0</v>
@@ -1355,7 +1355,7 @@
         <v>0</v>
       </c>
       <c r="H28">
-        <v>50</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1410,10 +1410,10 @@
         <v>39</v>
       </c>
       <c r="B2">
-        <v>60.2</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1421,10 +1421,10 @@
         <v>40</v>
       </c>
       <c r="B3">
-        <v>60.6</v>
+        <v>59.8</v>
       </c>
       <c r="C3">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1432,10 +1432,10 @@
         <v>41</v>
       </c>
       <c r="B4">
-        <v>60.8</v>
+        <v>60.3</v>
       </c>
       <c r="C4">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1443,10 +1443,10 @@
         <v>42</v>
       </c>
       <c r="B5">
-        <v>60.8</v>
+        <v>60.5</v>
       </c>
       <c r="C5">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1454,10 +1454,10 @@
         <v>43</v>
       </c>
       <c r="B6">
-        <v>87.2</v>
+        <v>60.5</v>
       </c>
       <c r="C6">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1465,10 +1465,10 @@
         <v>44</v>
       </c>
       <c r="B7">
-        <v>90.09999999999999</v>
+        <v>83.3</v>
       </c>
       <c r="C7">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1476,10 +1476,10 @@
         <v>45</v>
       </c>
       <c r="B8">
-        <v>94.90000000000001</v>
+        <v>90.3</v>
       </c>
       <c r="C8">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1487,10 +1487,10 @@
         <v>46</v>
       </c>
       <c r="B9">
-        <v>98</v>
+        <v>97.8</v>
       </c>
       <c r="C9">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1501,7 +1501,7 @@
         <v>98.5</v>
       </c>
       <c r="C10">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1512,7 +1512,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="C11">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1520,10 +1520,10 @@
         <v>49</v>
       </c>
       <c r="B12">
-        <v>99.90000000000001</v>
+        <v>99.8</v>
       </c>
       <c r="C12">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1534,7 +1534,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1545,7 +1545,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1556,7 +1556,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1567,7 +1567,7 @@
         <v>100</v>
       </c>
       <c r="C16">
-        <v>1361</v>
+        <v>1325</v>
       </c>
     </row>
   </sheetData>
@@ -1593,24 +1593,24 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2">
-        <v>402</v>
+        <v>394</v>
       </c>
       <c r="C2">
-        <v>29.5</v>
+        <v>29.7</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="C3">
-        <v>15.1</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1618,10 +1618,10 @@
         <v>57</v>
       </c>
       <c r="B4">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="C4">
-        <v>12.6</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1629,7 +1629,7 @@
         <v>58</v>
       </c>
       <c r="B5">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="C5">
         <v>11.8</v>
@@ -1640,7 +1640,7 @@
         <v>59</v>
       </c>
       <c r="B6">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C6">
         <v>10.9</v>
@@ -1651,7 +1651,7 @@
         <v>60</v>
       </c>
       <c r="B7">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C7">
         <v>3.5</v>
@@ -1659,18 +1659,18 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8">
         <v>34</v>
       </c>
       <c r="C8">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9">
         <v>27</v>
@@ -1684,7 +1684,7 @@
         <v>61</v>
       </c>
       <c r="B10">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C10">
         <v>0.8</v>
@@ -1698,7 +1698,7 @@
         <v>10</v>
       </c>
       <c r="C11">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>
@@ -1733,10 +1733,10 @@
         <v>128</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2">
-        <v>2.3</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1744,7 +1744,7 @@
         <v>66</v>
       </c>
       <c r="B3">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1758,7 +1758,7 @@
         <v>67</v>
       </c>
       <c r="B4">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1800,13 +1800,13 @@
         <v>70</v>
       </c>
       <c r="B7">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
       <c r="D7">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1814,7 +1814,7 @@
         <v>71</v>
       </c>
       <c r="B8">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1828,7 +1828,7 @@
         <v>72</v>
       </c>
       <c r="B9">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1842,13 +1842,13 @@
         <v>73</v>
       </c>
       <c r="B10">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D10">
-        <v>12.2</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -1856,7 +1856,7 @@
         <v>74</v>
       </c>
       <c r="B11">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1870,13 +1870,13 @@
         <v>75</v>
       </c>
       <c r="B12">
-        <v>602</v>
+        <v>580</v>
       </c>
       <c r="C12">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="D12">
-        <v>15.8</v>
+        <v>14.5</v>
       </c>
     </row>
   </sheetData>
@@ -1922,13 +1922,13 @@
         <v>66</v>
       </c>
       <c r="B3">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="C3">
         <v>45</v>
       </c>
       <c r="D3">
-        <v>19.9</v>
+        <v>20.3</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1936,13 +1936,13 @@
         <v>67</v>
       </c>
       <c r="B4">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C4">
         <v>5</v>
       </c>
       <c r="D4">
-        <v>16.1</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1978,13 +1978,13 @@
         <v>70</v>
       </c>
       <c r="B7">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D7">
-        <v>34.3</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1992,13 +1992,13 @@
         <v>71</v>
       </c>
       <c r="B8">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C8">
         <v>15</v>
       </c>
       <c r="D8">
-        <v>34.1</v>
+        <v>34.9</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2006,13 +2006,13 @@
         <v>72</v>
       </c>
       <c r="B9">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C9">
         <v>20</v>
       </c>
       <c r="D9">
-        <v>25.6</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2020,13 +2020,13 @@
         <v>73</v>
       </c>
       <c r="B10">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C10">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D10">
-        <v>33.8</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2034,13 +2034,13 @@
         <v>74</v>
       </c>
       <c r="B11">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C11">
         <v>28</v>
       </c>
       <c r="D11">
-        <v>24.3</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2048,13 +2048,13 @@
         <v>75</v>
       </c>
       <c r="B12">
-        <v>602</v>
+        <v>580</v>
       </c>
       <c r="C12">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="D12">
-        <v>28.4</v>
+        <v>27.4</v>
       </c>
     </row>
   </sheetData>
@@ -2083,10 +2083,10 @@
         <v>78</v>
       </c>
       <c r="B2">
-        <v>788</v>
+        <v>739</v>
       </c>
       <c r="C2">
-        <v>98.59999999999999</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2094,10 +2094,10 @@
         <v>79</v>
       </c>
       <c r="B3">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C3">
-        <v>1.1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2137,10 +2137,10 @@
         <v>82</v>
       </c>
       <c r="B2">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2148,10 +2148,10 @@
         <v>83</v>
       </c>
       <c r="B3">
-        <v>984</v>
+        <v>959</v>
       </c>
       <c r="C3">
-        <v>72.3</v>
+        <v>72.40000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2159,10 +2159,10 @@
         <v>84</v>
       </c>
       <c r="B4">
-        <v>350</v>
+        <v>337</v>
       </c>
       <c r="C4">
-        <v>25.7</v>
+        <v>25.4</v>
       </c>
     </row>
   </sheetData>
@@ -2194,7 +2194,7 @@
         <v>2</v>
       </c>
       <c r="C2">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2202,10 +2202,10 @@
         <v>86</v>
       </c>
       <c r="B3">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="C3">
-        <v>40</v>
+        <v>40.5</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2213,10 +2213,10 @@
         <v>87</v>
       </c>
       <c r="B4">
-        <v>815</v>
+        <v>787</v>
       </c>
       <c r="C4">
-        <v>59.9</v>
+        <v>59.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização de dados — 19/09/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="87">
   <si>
     <t>municipio</t>
   </si>
@@ -50,13 +50,16 @@
     <t>Nova Esperanca</t>
   </si>
   <si>
+    <t>Santa Ines</t>
+  </si>
+  <si>
     <t>Uniflor</t>
   </si>
   <si>
     <t>Ourizona</t>
   </si>
   <si>
-    <t>Santa Ines</t>
+    <t>Sao Jorge Do Ivai</t>
   </si>
   <si>
     <t>Atalaia</t>
@@ -68,9 +71,6 @@
     <t>Nossa Senhora Das Gracas</t>
   </si>
   <si>
-    <t>Sao Jorge Do Ivai</t>
-  </si>
-  <si>
     <t>Maringa</t>
   </si>
   <si>
@@ -80,12 +80,12 @@
     <t>Colorado</t>
   </si>
   <si>
+    <t>Florai</t>
+  </si>
+  <si>
     <t>Itambe</t>
   </si>
   <si>
-    <t>Florai</t>
-  </si>
-  <si>
     <t>Marialva</t>
   </si>
   <si>
@@ -95,30 +95,30 @@
     <t>Sarandi</t>
   </si>
   <si>
+    <t>Munhoz De Melo</t>
+  </si>
+  <si>
+    <t>Lobato</t>
+  </si>
+  <si>
     <t>Astorga</t>
   </si>
   <si>
     <t>Floresta</t>
   </si>
   <si>
-    <t>Munhoz De Melo</t>
+    <t>Paicandu</t>
   </si>
   <si>
     <t>Mandaguacu</t>
   </si>
   <si>
-    <t>Paicandu</t>
-  </si>
-  <si>
     <t>Presidente Castelo Branco</t>
   </si>
   <si>
     <t>Santa Fe</t>
   </si>
   <si>
-    <t>Lobato</t>
-  </si>
-  <si>
     <t>Florida</t>
   </si>
   <si>
@@ -143,30 +143,27 @@
     <t>Obesidade</t>
   </si>
   <si>
+    <t>Cardiopatia</t>
+  </si>
+  <si>
     <t>Diabetes</t>
   </si>
   <si>
-    <t>Cardiopatia</t>
-  </si>
-  <si>
     <t>Imunodepressão</t>
   </si>
   <si>
     <t>Evolução (Desfecho)</t>
   </si>
   <si>
-    <t>Bairro</t>
-  </si>
-  <si>
     <t>Critério Confirmação</t>
   </si>
   <si>
+    <t>Raça/Cor</t>
+  </si>
+  <si>
     <t>Antiviral</t>
   </si>
   <si>
-    <t>Raça/Cor</t>
-  </si>
-  <si>
     <t>Data Internação</t>
   </si>
   <si>
@@ -206,10 +203,10 @@
     <t>Doença Renal</t>
   </si>
   <si>
+    <t>Síndrome de Down</t>
+  </si>
+  <si>
     <t>Doença Hepática</t>
-  </si>
-  <si>
-    <t>Síndrome de Down</t>
   </si>
   <si>
     <t>faixa_etaria</t>
@@ -661,25 +658,25 @@
         <v>8</v>
       </c>
       <c r="B2">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2">
-        <v>364.7</v>
+        <v>372.1</v>
       </c>
       <c r="F2">
-        <v>36.8</v>
+        <v>33.2</v>
       </c>
       <c r="G2">
-        <v>10.1</v>
+        <v>8.9</v>
       </c>
       <c r="H2">
-        <v>5.1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -687,22 +684,22 @@
         <v>9</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3">
-        <v>284.9</v>
+        <v>286.5</v>
       </c>
       <c r="F3">
-        <v>47.5</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>16.7</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -713,25 +710,25 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>250.5</v>
+        <v>284.9</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>47.5</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>16.7</v>
       </c>
       <c r="H4">
-        <v>37.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -739,16 +736,16 @@
         <v>11</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E5">
-        <v>229.2</v>
+        <v>250.5</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -757,7 +754,7 @@
         <v>0</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -765,16 +762,16 @@
         <v>12</v>
       </c>
       <c r="B6">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E6">
-        <v>222.4</v>
+        <v>232.1</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -783,7 +780,7 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -791,25 +788,25 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>220.8</v>
+        <v>222.4</v>
       </c>
       <c r="F7">
-        <v>22.1</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -817,25 +814,25 @@
         <v>14</v>
       </c>
       <c r="B8">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8">
-        <v>218</v>
+        <v>220.8</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>22.1</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H8">
-        <v>37.5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -843,25 +840,25 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9">
         <v>3</v>
       </c>
       <c r="E9">
-        <v>212.8</v>
+        <v>218</v>
       </c>
       <c r="F9">
-        <v>19.3</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>9.1</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>27.3</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -869,25 +866,25 @@
         <v>16</v>
       </c>
       <c r="B10">
-        <v>863</v>
+        <v>907</v>
       </c>
       <c r="C10">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="D10">
-        <v>244</v>
+        <v>261</v>
       </c>
       <c r="E10">
-        <v>200.9</v>
+        <v>211.1</v>
       </c>
       <c r="F10">
-        <v>20.2</v>
+        <v>16.8</v>
       </c>
       <c r="G10">
-        <v>10.1</v>
+        <v>7.9</v>
       </c>
       <c r="H10">
-        <v>28.3</v>
+        <v>28.8</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -947,7 +944,7 @@
         <v>19</v>
       </c>
       <c r="B13">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -956,7 +953,7 @@
         <v>2</v>
       </c>
       <c r="E13">
-        <v>160.6</v>
+        <v>145.7</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -965,7 +962,7 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>20</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -973,7 +970,7 @@
         <v>20</v>
       </c>
       <c r="B14">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -982,7 +979,7 @@
         <v>2</v>
       </c>
       <c r="E14">
-        <v>145.7</v>
+        <v>144.5</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -991,7 +988,7 @@
         <v>0</v>
       </c>
       <c r="H14">
-        <v>28.6</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -999,25 +996,25 @@
         <v>21</v>
       </c>
       <c r="B15">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C15">
         <v>2</v>
       </c>
       <c r="D15">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E15">
-        <v>129.6</v>
+        <v>138.6</v>
       </c>
       <c r="F15">
         <v>4.5</v>
       </c>
       <c r="G15">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="H15">
-        <v>46.6</v>
+        <v>46.8</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1051,25 +1048,25 @@
         <v>23</v>
       </c>
       <c r="B17">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C17">
         <v>8</v>
       </c>
       <c r="D17">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E17">
-        <v>89</v>
+        <v>95.2</v>
       </c>
       <c r="F17">
         <v>6.2</v>
       </c>
       <c r="G17">
-        <v>7</v>
+        <v>6.6</v>
       </c>
       <c r="H17">
-        <v>39.5</v>
+        <v>39.3</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1077,25 +1074,25 @@
         <v>24</v>
       </c>
       <c r="B18">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
         <v>1</v>
       </c>
-      <c r="D18">
-        <v>5</v>
-      </c>
       <c r="E18">
-        <v>53.4</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="F18">
-        <v>3.8</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>7.1</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>35.7</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1103,7 +1100,7 @@
         <v>25</v>
       </c>
       <c r="B19">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1112,7 +1109,7 @@
         <v>1</v>
       </c>
       <c r="E19">
-        <v>52.1</v>
+        <v>63.7</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -1121,7 +1118,7 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>16.7</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1129,16 +1126,16 @@
         <v>26</v>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E20">
-        <v>49.3</v>
+        <v>57.2</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -1147,7 +1144,7 @@
         <v>0</v>
       </c>
       <c r="H20">
-        <v>50</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1155,16 +1152,16 @@
         <v>27</v>
       </c>
       <c r="B21">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E21">
-        <v>49.2</v>
+        <v>52.1</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -1173,7 +1170,7 @@
         <v>0</v>
       </c>
       <c r="H21">
-        <v>41.2</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1181,25 +1178,25 @@
         <v>28</v>
       </c>
       <c r="B22">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C22">
         <v>1</v>
       </c>
       <c r="D22">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E22">
-        <v>47.2</v>
+        <v>49.3</v>
       </c>
       <c r="F22">
         <v>2.1</v>
       </c>
       <c r="G22">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="H22">
-        <v>60.9</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1207,25 +1204,25 @@
         <v>29</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="C23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E23">
-        <v>46.5</v>
+        <v>49.2</v>
       </c>
       <c r="F23">
-        <v>23.2</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>41.2</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1233,25 +1230,25 @@
         <v>30</v>
       </c>
       <c r="B24">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D24">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E24">
-        <v>42.6</v>
+        <v>46.5</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>23.2</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H24">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1259,16 +1256,16 @@
         <v>31</v>
       </c>
       <c r="B25">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E25">
-        <v>42.5</v>
+        <v>42.6</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1277,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1391,7 +1388,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1410,10 +1407,10 @@
         <v>39</v>
       </c>
       <c r="B2">
-        <v>60.2</v>
+        <v>61.2</v>
       </c>
       <c r="C2">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1421,10 +1418,10 @@
         <v>40</v>
       </c>
       <c r="B3">
-        <v>60.6</v>
+        <v>61.7</v>
       </c>
       <c r="C3">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1432,10 +1429,10 @@
         <v>41</v>
       </c>
       <c r="B4">
-        <v>60.8</v>
+        <v>61.7</v>
       </c>
       <c r="C4">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1443,10 +1440,10 @@
         <v>42</v>
       </c>
       <c r="B5">
-        <v>60.8</v>
+        <v>61.7</v>
       </c>
       <c r="C5">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1454,10 +1451,10 @@
         <v>43</v>
       </c>
       <c r="B6">
-        <v>87.2</v>
+        <v>88.7</v>
       </c>
       <c r="C6">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1465,10 +1462,10 @@
         <v>44</v>
       </c>
       <c r="B7">
-        <v>90.09999999999999</v>
+        <v>95</v>
       </c>
       <c r="C7">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1476,10 +1473,10 @@
         <v>45</v>
       </c>
       <c r="B8">
-        <v>94.90000000000001</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="C8">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1487,10 +1484,10 @@
         <v>46</v>
       </c>
       <c r="B9">
-        <v>98</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="C9">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1498,10 +1495,10 @@
         <v>47</v>
       </c>
       <c r="B10">
-        <v>98.5</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="C10">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1509,10 +1506,10 @@
         <v>48</v>
       </c>
       <c r="B11">
-        <v>98.90000000000001</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="C11">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1520,10 +1517,10 @@
         <v>49</v>
       </c>
       <c r="B12">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="C12">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1534,7 +1531,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1545,7 +1542,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1556,18 +1553,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1361</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16">
-        <v>100</v>
-      </c>
-      <c r="C16">
-        <v>1361</v>
+        <v>1424</v>
       </c>
     </row>
   </sheetData>
@@ -1582,79 +1568,79 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
-        <v>402</v>
+        <v>435</v>
       </c>
       <c r="C2">
-        <v>29.5</v>
+        <v>30.5</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="C3">
-        <v>15.1</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B4">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C4">
-        <v>12.6</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="C5">
-        <v>11.8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C6">
-        <v>10.9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C7">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1662,10 +1648,10 @@
         <v>39</v>
       </c>
       <c r="B8">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C8">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1676,15 +1662,15 @@
         <v>27</v>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B10">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C10">
         <v>0.8</v>
@@ -1692,7 +1678,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -1713,13 +1699,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>6</v>
@@ -1727,24 +1713,24 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B2">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C2">
+        <v>4</v>
+      </c>
+      <c r="D2">
         <v>3</v>
-      </c>
-      <c r="D2">
-        <v>2.3</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B3">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1755,10 +1741,10 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B4">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1769,21 +1755,21 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
       <c r="D5">
-        <v>28.6</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B6">
         <v>21</v>
@@ -1797,7 +1783,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B7">
         <v>35</v>
@@ -1811,52 +1797,52 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B8">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>2.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B9">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B10">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="C10">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D10">
-        <v>12.2</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B11">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1867,16 +1853,16 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B12">
-        <v>602</v>
+        <v>632</v>
       </c>
       <c r="C12">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="D12">
-        <v>15.8</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1891,7 +1877,7 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1905,63 +1891,63 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B2">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C2">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D2">
-        <v>44.5</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B3">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="C3">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D3">
-        <v>19.9</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B4">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4">
         <v>5</v>
       </c>
       <c r="D4">
-        <v>16.1</v>
+        <v>15.6</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>28.6</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B6">
         <v>21</v>
@@ -1975,7 +1961,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B7">
         <v>35</v>
@@ -1989,72 +1975,72 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B8">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C8">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D8">
-        <v>34.1</v>
+        <v>36.2</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B9">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C9">
         <v>20</v>
       </c>
       <c r="D9">
-        <v>25.6</v>
+        <v>24.4</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B10">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="C10">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D10">
-        <v>33.8</v>
+        <v>34.6</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B11">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C11">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D11">
-        <v>24.3</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B12">
-        <v>602</v>
+        <v>632</v>
       </c>
       <c r="C12">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D12">
-        <v>28.4</v>
+        <v>27.8</v>
       </c>
     </row>
   </sheetData>
@@ -2069,46 +2055,46 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>77</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B2">
-        <v>788</v>
+        <v>822</v>
       </c>
       <c r="C2">
-        <v>98.59999999999999</v>
+        <v>98.90000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C3">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -2123,46 +2109,46 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B2">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B3">
-        <v>984</v>
+        <v>1031</v>
       </c>
       <c r="C3">
-        <v>72.3</v>
+        <v>72.40000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B4">
-        <v>350</v>
+        <v>373</v>
       </c>
       <c r="C4">
-        <v>25.7</v>
+        <v>26.2</v>
       </c>
     </row>
   </sheetData>
@@ -2177,18 +2163,18 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -2199,24 +2185,24 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B3">
-        <v>544</v>
+        <v>568</v>
       </c>
       <c r="C3">
-        <v>40</v>
+        <v>39.9</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B4">
-        <v>815</v>
+        <v>854</v>
       </c>
       <c r="C4">
-        <v>59.9</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>